<commit_message>
Aggiungi secondo blocco listino prodotti (115 voci)
Naturaltech, OI, Pasta & Love, Heart of Glass, More Inside e le due
maschere Circle mancanti. Totale prodotti a listino: 216.

Applicati i due prezzi corretti a penna sul depliant:
Energizing Shampoo 250 ml (22,90 -> 23,00) e Energizing Superactive
Anytime 100 ml (82,00 -> 85,00), entrambi da confermare.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HaLJpnaiiT1t5t7Nsc7fzN
</commit_message>
<xml_diff>
--- a/registro_giornaliero.xlsx
+++ b/registro_giornaliero.xlsx
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E110"/>
+  <dimension ref="A1:E225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2946,6 +2946,2421 @@
         <v>9.5</v>
       </c>
       <c r="E110" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="7" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t>The Let It Go Circle 50 ml</t>
+        </is>
+      </c>
+      <c r="C111" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Circle Chronicles</t>
+        </is>
+      </c>
+      <c r="D111" s="8" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E111" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="7" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="7" t="inlineStr">
+        <is>
+          <t>The Restless Circle 50 ml</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Circle Chronicles</t>
+        </is>
+      </c>
+      <c r="D112" s="8" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E112" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="7" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t>Renewing Shampoo 100 ml</t>
+        </is>
+      </c>
+      <c r="C113" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D113" s="8" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="E113" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="7" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="7" t="inlineStr">
+        <is>
+          <t>Renewing Shampoo 250 ml</t>
+        </is>
+      </c>
+      <c r="C114" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D114" s="8" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E114" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="7" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>Renewing Shampoo 1000 ml</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D115" s="8" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="E115" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="7" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="7" t="inlineStr">
+        <is>
+          <t>Renewing Conditioning Treatment 60 ml</t>
+        </is>
+      </c>
+      <c r="C116" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D116" s="8" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="E116" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="7" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t>Renewing Conditioning Treatment 250 ml</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D117" s="8" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="E117" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="7" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="7" t="inlineStr">
+        <is>
+          <t>Renewing Conditioning Treatment 1000 ml</t>
+        </is>
+      </c>
+      <c r="C118" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D118" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E118" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="7" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="7" t="inlineStr">
+        <is>
+          <t>Replumping Shampoo 100 ml</t>
+        </is>
+      </c>
+      <c r="C119" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D119" s="8" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="E119" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="7" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="7" t="inlineStr">
+        <is>
+          <t>Replumping Shampoo 250 ml</t>
+        </is>
+      </c>
+      <c r="C120" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D120" s="8" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E120" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t>Replumping Shampoo 1000 ml</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D121" s="8" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="E121" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="7" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="7" t="inlineStr">
+        <is>
+          <t>Replumping Conditioner 60 ml</t>
+        </is>
+      </c>
+      <c r="C122" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D122" s="8" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="E122" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="7" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="7" t="inlineStr">
+        <is>
+          <t>Replumping Conditioner 150 ml</t>
+        </is>
+      </c>
+      <c r="C123" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D123" s="8" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="E123" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="7" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="7" t="inlineStr">
+        <is>
+          <t>Replumping Conditioner 1000 ml</t>
+        </is>
+      </c>
+      <c r="C124" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D124" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E124" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="7" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="7" t="inlineStr">
+        <is>
+          <t>Replumping Hair Filler Superactive 100 ml</t>
+        </is>
+      </c>
+      <c r="C125" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D125" s="8" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="E125" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="7" t="inlineStr">
+        <is>
+          <t>Energizing Shampoo 100 ml</t>
+        </is>
+      </c>
+      <c r="C126" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D126" s="8" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="E126" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="7" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="7" t="inlineStr">
+        <is>
+          <t>Energizing Shampoo 250 ml</t>
+        </is>
+      </c>
+      <c r="C127" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D127" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="E127" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="7" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="7" t="inlineStr">
+        <is>
+          <t>Energizing Shampoo 1000 ml</t>
+        </is>
+      </c>
+      <c r="C128" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D128" s="8" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="E128" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="7" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="7" t="inlineStr">
+        <is>
+          <t>Energizing Seasonal Superactive 100 ml</t>
+        </is>
+      </c>
+      <c r="C129" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D129" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="E129" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="7" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="7" t="inlineStr">
+        <is>
+          <t>Energizing Seasonal Superactive 12x6 ml</t>
+        </is>
+      </c>
+      <c r="C130" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D130" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="E130" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="7" t="inlineStr">
+        <is>
+          <t>Energizing Superactive Anytime 100 ml</t>
+        </is>
+      </c>
+      <c r="C131" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D131" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="E131" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="7" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="7" t="inlineStr">
+        <is>
+          <t>Energizing Gel 150 ml</t>
+        </is>
+      </c>
+      <c r="C132" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D132" s="8" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="E132" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="7" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="7" t="inlineStr">
+        <is>
+          <t>Energizing Thickening Tonic 100 ml</t>
+        </is>
+      </c>
+      <c r="C133" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D133" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="E133" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="7" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="7" t="inlineStr">
+        <is>
+          <t>Purifying Shampoo 100 ml</t>
+        </is>
+      </c>
+      <c r="C134" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D134" s="8" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="E134" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="7" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="7" t="inlineStr">
+        <is>
+          <t>Purifying Shampoo 250 ml</t>
+        </is>
+      </c>
+      <c r="C135" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D135" s="8" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E135" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="7" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="7" t="inlineStr">
+        <is>
+          <t>Purifying Shampoo 1000 ml</t>
+        </is>
+      </c>
+      <c r="C136" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D136" s="8" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="E136" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="7" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="7" t="inlineStr">
+        <is>
+          <t>Purifying Gel 150 ml</t>
+        </is>
+      </c>
+      <c r="C137" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="E137" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="7" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="7" t="inlineStr">
+        <is>
+          <t>Well-Being Shampoo 100 ml</t>
+        </is>
+      </c>
+      <c r="C138" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D138" s="8" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="E138" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="7" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="7" t="inlineStr">
+        <is>
+          <t>Well-Being Shampoo 250 ml</t>
+        </is>
+      </c>
+      <c r="C139" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D139" s="8" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E139" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="7" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="7" t="inlineStr">
+        <is>
+          <t>Well-Being Shampoo 1000 ml</t>
+        </is>
+      </c>
+      <c r="C140" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D140" s="8" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="E140" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="7" t="inlineStr">
+        <is>
+          <t>Well-Being Conditioner 60 ml</t>
+        </is>
+      </c>
+      <c r="C141" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D141" s="8" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="E141" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="7" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="7" t="inlineStr">
+        <is>
+          <t>Well-Being Conditioner 150 ml</t>
+        </is>
+      </c>
+      <c r="C142" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D142" s="8" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="E142" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="7" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="7" t="inlineStr">
+        <is>
+          <t>Well-Being Conditioner 1000 ml</t>
+        </is>
+      </c>
+      <c r="C143" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D143" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E143" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="7" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="7" t="inlineStr">
+        <is>
+          <t>Detoxifying Scrub Shampoo 100 ml</t>
+        </is>
+      </c>
+      <c r="C144" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D144" s="8" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="E144" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="7" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="7" t="inlineStr">
+        <is>
+          <t>Detoxifying Scrub Shampoo 250 ml</t>
+        </is>
+      </c>
+      <c r="C145" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D145" s="8" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E145" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="7" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="7" t="inlineStr">
+        <is>
+          <t>Detoxifying Scrub Shampoo 1000 ml</t>
+        </is>
+      </c>
+      <c r="C146" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D146" s="8" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="E146" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="7" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="7" t="inlineStr">
+        <is>
+          <t>Rebalancing Shampoo 100 ml</t>
+        </is>
+      </c>
+      <c r="C147" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D147" s="8" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="E147" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="7" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="7" t="inlineStr">
+        <is>
+          <t>Rebalancing Shampoo 250 ml</t>
+        </is>
+      </c>
+      <c r="C148" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D148" s="8" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E148" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="7" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="7" t="inlineStr">
+        <is>
+          <t>Rebalancing Shampoo 1000 ml</t>
+        </is>
+      </c>
+      <c r="C149" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D149" s="8" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="E149" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="7" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" s="7" t="inlineStr">
+        <is>
+          <t>Cleansing Treatment 250 ml</t>
+        </is>
+      </c>
+      <c r="C150" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D150" s="8" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="E150" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" s="7" t="inlineStr">
+        <is>
+          <t>Cleansing Treatment 1000 ml</t>
+        </is>
+      </c>
+      <c r="C151" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D151" s="8" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="E151" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="7" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" s="7" t="inlineStr">
+        <is>
+          <t>Calming Shampoo 100 ml</t>
+        </is>
+      </c>
+      <c r="C152" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D152" s="8" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="E152" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="7" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" s="7" t="inlineStr">
+        <is>
+          <t>Calming Shampoo 250 ml</t>
+        </is>
+      </c>
+      <c r="C153" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D153" s="8" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E153" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="7" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" s="7" t="inlineStr">
+        <is>
+          <t>Calming Shampoo 1000 ml</t>
+        </is>
+      </c>
+      <c r="C154" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D154" s="8" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="E154" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="7" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" s="7" t="inlineStr">
+        <is>
+          <t>Calming Superactive 100 ml</t>
+        </is>
+      </c>
+      <c r="C155" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D155" s="8" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="E155" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="7" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Shampoo 100 ml</t>
+        </is>
+      </c>
+      <c r="C156" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D156" s="8" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="E156" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="7" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Shampoo 250 ml</t>
+        </is>
+      </c>
+      <c r="C157" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D157" s="8" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E157" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="7" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Shampoo 1000 ml</t>
+        </is>
+      </c>
+      <c r="C158" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D158" s="8" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="E158" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="7" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Vegetarian Miracle Conditioner 60 ml</t>
+        </is>
+      </c>
+      <c r="C159" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D159" s="8" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="E159" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="7" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Vegetarian Miracle Conditioner 250 ml</t>
+        </is>
+      </c>
+      <c r="C160" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D160" s="8" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="E160" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="7" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Vegetarian Miracle Conditioner 1000 ml</t>
+        </is>
+      </c>
+      <c r="C161" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D161" s="8" t="n">
+        <v>113.4</v>
+      </c>
+      <c r="E161" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="7" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Vegetarian Miracle Mask 60 ml</t>
+        </is>
+      </c>
+      <c r="C162" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D162" s="8" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E162" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="7" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Vegetarian Miracle Mask 250 ml</t>
+        </is>
+      </c>
+      <c r="C163" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D163" s="8" t="n">
+        <v>43</v>
+      </c>
+      <c r="E163" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="7" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Vegetarian Miracle Mask 1000 ml</t>
+        </is>
+      </c>
+      <c r="C164" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D164" s="8" t="n">
+        <v>129</v>
+      </c>
+      <c r="E164" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="7" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Hair Building Pak 60 ml</t>
+        </is>
+      </c>
+      <c r="C165" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D165" s="8" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="E165" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="7" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Hair Building Pak 250 ml</t>
+        </is>
+      </c>
+      <c r="C166" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D166" s="8" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="E166" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="7" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Keratin Sealer 100 ml</t>
+        </is>
+      </c>
+      <c r="C167" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D167" s="8" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="E167" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="7" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" s="7" t="inlineStr">
+        <is>
+          <t>Nourishing Hair Royal Jelly Superactive 6x8 ml</t>
+        </is>
+      </c>
+      <c r="C168" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D168" s="8" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="E168" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="7" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" s="7" t="inlineStr">
+        <is>
+          <t>Elevating Scalp Recovery Treatment 100 ml</t>
+        </is>
+      </c>
+      <c r="C169" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Naturaltech</t>
+        </is>
+      </c>
+      <c r="D169" s="8" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="E169" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="7" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" s="7" t="inlineStr">
+        <is>
+          <t>OI/Shampoo 90 ml</t>
+        </is>
+      </c>
+      <c r="C170" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D170" s="8" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="E170" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="7" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" s="7" t="inlineStr">
+        <is>
+          <t>OI/Shampoo 280 ml</t>
+        </is>
+      </c>
+      <c r="C171" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D171" s="8" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="E171" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="7" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" s="7" t="inlineStr">
+        <is>
+          <t>OI/Shampoo 1000 ml</t>
+        </is>
+      </c>
+      <c r="C172" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D172" s="8" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="E172" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="7" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" s="7" t="inlineStr">
+        <is>
+          <t>OI/Conditioner 75 ml</t>
+        </is>
+      </c>
+      <c r="C173" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D173" s="8" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="E173" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="7" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" s="7" t="inlineStr">
+        <is>
+          <t>OI/Conditioner 250 ml</t>
+        </is>
+      </c>
+      <c r="C174" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D174" s="8" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="E174" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="7" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" s="7" t="inlineStr">
+        <is>
+          <t>OI/Conditioner 1000 ml</t>
+        </is>
+      </c>
+      <c r="C175" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D175" s="8" t="n">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="E175" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="7" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" s="7" t="inlineStr">
+        <is>
+          <t>OI/Hair Butter 75 ml</t>
+        </is>
+      </c>
+      <c r="C176" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D176" s="8" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="E176" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="7" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" s="7" t="inlineStr">
+        <is>
+          <t>OI/Hair Butter 250 ml</t>
+        </is>
+      </c>
+      <c r="C177" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D177" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="E177" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="7" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" s="7" t="inlineStr">
+        <is>
+          <t>OI/Hair Butter 1000 ml</t>
+        </is>
+      </c>
+      <c r="C178" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D178" s="8" t="n">
+        <v>102</v>
+      </c>
+      <c r="E178" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="7" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" s="7" t="inlineStr">
+        <is>
+          <t>OI/Oil 50 ml</t>
+        </is>
+      </c>
+      <c r="C179" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D179" s="8" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="E179" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="7" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" s="7" t="inlineStr">
+        <is>
+          <t>OI/Oil 135 ml</t>
+        </is>
+      </c>
+      <c r="C180" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D180" s="8" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="E180" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="7" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" s="7" t="inlineStr">
+        <is>
+          <t>OI/Liquid Luster 100 ml</t>
+        </is>
+      </c>
+      <c r="C181" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D181" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="E181" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="7" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" s="7" t="inlineStr">
+        <is>
+          <t>OI/Liquid Luster 300 ml</t>
+        </is>
+      </c>
+      <c r="C182" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D182" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="E182" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="7" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" s="7" t="inlineStr">
+        <is>
+          <t>OI/All in One Milk 50 ml</t>
+        </is>
+      </c>
+      <c r="C183" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D183" s="8" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="E183" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="7" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" s="7" t="inlineStr">
+        <is>
+          <t>OI/All in One Milk 135 ml</t>
+        </is>
+      </c>
+      <c r="C184" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D184" s="8" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="E184" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="7" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" s="7" t="inlineStr">
+        <is>
+          <t>OI/Body Wash 90 ml</t>
+        </is>
+      </c>
+      <c r="C185" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D185" s="8" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E185" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="7" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" s="7" t="inlineStr">
+        <is>
+          <t>OI/Body Wash 280 ml</t>
+        </is>
+      </c>
+      <c r="C186" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D186" s="8" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="E186" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="7" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" s="7" t="inlineStr">
+        <is>
+          <t>OI/Hand Balm 75 ml</t>
+        </is>
+      </c>
+      <c r="C187" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - OI</t>
+        </is>
+      </c>
+      <c r="D187" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="E187" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="7" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" s="7" t="inlineStr">
+        <is>
+          <t>Softening Shaving Gel 200 ml</t>
+        </is>
+      </c>
+      <c r="C188" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Pasta &amp; Love</t>
+        </is>
+      </c>
+      <c r="D188" s="8" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="E188" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="7" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" s="7" t="inlineStr">
+        <is>
+          <t>After Shave &amp; Moisturizing Cream 100 ml</t>
+        </is>
+      </c>
+      <c r="C189" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Pasta &amp; Love</t>
+        </is>
+      </c>
+      <c r="D189" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="E189" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="7" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" s="7" t="inlineStr">
+        <is>
+          <t>Pre-Shaving &amp; Beard Oil 50 ml</t>
+        </is>
+      </c>
+      <c r="C190" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Pasta &amp; Love</t>
+        </is>
+      </c>
+      <c r="D190" s="8" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="E190" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="7" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" s="7" t="inlineStr">
+        <is>
+          <t>Medium Hold Styling Paste 125 ml</t>
+        </is>
+      </c>
+      <c r="C191" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Pasta &amp; Love</t>
+        </is>
+      </c>
+      <c r="D191" s="8" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="E191" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="7" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" s="7" t="inlineStr">
+        <is>
+          <t>Non-Foaming Transparent Shaving Gel 150 ml</t>
+        </is>
+      </c>
+      <c r="C192" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Pasta &amp; Love</t>
+        </is>
+      </c>
+      <c r="D192" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="E192" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="7" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" s="7" t="inlineStr">
+        <is>
+          <t>Strong-Hold Mat Clay 50 ml</t>
+        </is>
+      </c>
+      <c r="C193" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Pasta &amp; Love</t>
+        </is>
+      </c>
+      <c r="D193" s="8" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="E193" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="7" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" s="7" t="inlineStr">
+        <is>
+          <t>Hair Beard &amp; Body Wash 300 ml</t>
+        </is>
+      </c>
+      <c r="C194" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Pasta &amp; Love</t>
+        </is>
+      </c>
+      <c r="D194" s="8" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="E194" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="7" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" s="7" t="inlineStr">
+        <is>
+          <t>Fiber Cream 50 ml</t>
+        </is>
+      </c>
+      <c r="C195" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Pasta &amp; Love</t>
+        </is>
+      </c>
+      <c r="D195" s="8" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E195" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="7" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" s="7" t="inlineStr">
+        <is>
+          <t>Silkening Shampoo 90 ml</t>
+        </is>
+      </c>
+      <c r="C196" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Heart of Glass</t>
+        </is>
+      </c>
+      <c r="D196" s="8" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="E196" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="7" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" s="7" t="inlineStr">
+        <is>
+          <t>Silkening Shampoo 250 ml</t>
+        </is>
+      </c>
+      <c r="C197" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Heart of Glass</t>
+        </is>
+      </c>
+      <c r="D197" s="8" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="E197" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="7" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" s="7" t="inlineStr">
+        <is>
+          <t>Silkening Shampoo 1000 ml</t>
+        </is>
+      </c>
+      <c r="C198" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Heart of Glass</t>
+        </is>
+      </c>
+      <c r="D198" s="8" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="E198" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="7" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" s="7" t="inlineStr">
+        <is>
+          <t>Rich Conditioner 90 ml</t>
+        </is>
+      </c>
+      <c r="C199" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Heart of Glass</t>
+        </is>
+      </c>
+      <c r="D199" s="8" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="E199" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="7" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" s="7" t="inlineStr">
+        <is>
+          <t>Rich Conditioner 250 ml</t>
+        </is>
+      </c>
+      <c r="C200" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Heart of Glass</t>
+        </is>
+      </c>
+      <c r="D200" s="8" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="E200" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" s="7" t="inlineStr">
+        <is>
+          <t>Rich Conditioner 1000 ml</t>
+        </is>
+      </c>
+      <c r="C201" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Heart of Glass</t>
+        </is>
+      </c>
+      <c r="D201" s="8" t="n">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="E201" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="7" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" s="7" t="inlineStr">
+        <is>
+          <t>Intense Treatment 150 ml</t>
+        </is>
+      </c>
+      <c r="C202" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Heart of Glass</t>
+        </is>
+      </c>
+      <c r="D202" s="8" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="E202" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="7" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" s="7" t="inlineStr">
+        <is>
+          <t>Sheer Glaze 150 ml</t>
+        </is>
+      </c>
+      <c r="C203" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Heart of Glass</t>
+        </is>
+      </c>
+      <c r="D203" s="8" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="E203" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="7" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" s="7" t="inlineStr">
+        <is>
+          <t>Instant Bonding Glow 300 ml</t>
+        </is>
+      </c>
+      <c r="C204" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Heart of Glass</t>
+        </is>
+      </c>
+      <c r="D204" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="E204" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="7" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" s="7" t="inlineStr">
+        <is>
+          <t>Spray al Sale Marino 100 ml</t>
+        </is>
+      </c>
+      <c r="C205" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D205" s="8" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="E205" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="7" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" s="7" t="inlineStr">
+        <is>
+          <t>Spray al Sale Marino 250 ml</t>
+        </is>
+      </c>
+      <c r="C206" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D206" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="E206" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="7" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" s="7" t="inlineStr">
+        <is>
+          <t>Siero Crea Ricci 100 ml</t>
+        </is>
+      </c>
+      <c r="C207" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D207" s="8" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="E207" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="7" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" s="7" t="inlineStr">
+        <is>
+          <t>Siero Crea Ricci 250 ml</t>
+        </is>
+      </c>
+      <c r="C208" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D208" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="E208" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="7" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" s="7" t="inlineStr">
+        <is>
+          <t>Oil Non Oil 250 ml</t>
+        </is>
+      </c>
+      <c r="C209" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D209" s="8" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="E209" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="7" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" s="7" t="inlineStr">
+        <is>
+          <t>Gel Medio Modellante 250 ml</t>
+        </is>
+      </c>
+      <c r="C210" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D210" s="8" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="E210" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="B211" s="7" t="inlineStr">
+        <is>
+          <t>Gel Oil per i Ricci 250 ml</t>
+        </is>
+      </c>
+      <c r="C211" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D211" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="E211" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="7" t="n">
+        <v>211</v>
+      </c>
+      <c r="B212" s="7" t="inlineStr">
+        <is>
+          <t>Blow Dry Primer 100 ml</t>
+        </is>
+      </c>
+      <c r="C212" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D212" s="8" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="E212" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="7" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" s="7" t="inlineStr">
+        <is>
+          <t>Blow Dry Primer 250 ml</t>
+        </is>
+      </c>
+      <c r="C213" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D213" s="8" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="E213" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="7" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" s="7" t="inlineStr">
+        <is>
+          <t>Siero Texturizzante 150 ml</t>
+        </is>
+      </c>
+      <c r="C214" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D214" s="8" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="E214" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="7" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" s="7" t="inlineStr">
+        <is>
+          <t>Polvere Texturizzante 8 gr</t>
+        </is>
+      </c>
+      <c r="C215" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D215" s="8" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="E215" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="7" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" s="7" t="inlineStr">
+        <is>
+          <t>Siero Invisibile 50 ml</t>
+        </is>
+      </c>
+      <c r="C216" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D216" s="8" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="E216" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="7" t="n">
+        <v>216</v>
+      </c>
+      <c r="B217" s="7" t="inlineStr">
+        <is>
+          <t>Fluido Stirante Idratante 125 ml</t>
+        </is>
+      </c>
+      <c r="C217" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D217" s="8" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="E217" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="7" t="n">
+        <v>217</v>
+      </c>
+      <c r="B218" s="7" t="inlineStr">
+        <is>
+          <t>Crema Gel Forte 125 ml</t>
+        </is>
+      </c>
+      <c r="C218" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D218" s="8" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="E218" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="7" t="n">
+        <v>218</v>
+      </c>
+      <c r="B219" s="7" t="inlineStr">
+        <is>
+          <t>Pasta Duttile Media 125 ml</t>
+        </is>
+      </c>
+      <c r="C219" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D219" s="8" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="E219" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="7" t="n">
+        <v>219</v>
+      </c>
+      <c r="B220" s="7" t="inlineStr">
+        <is>
+          <t>Lacca Media 400 ml</t>
+        </is>
+      </c>
+      <c r="C220" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D220" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="E220" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="7" t="n">
+        <v>220</v>
+      </c>
+      <c r="B221" s="7" t="inlineStr">
+        <is>
+          <t>Lacca Forte 100 ml</t>
+        </is>
+      </c>
+      <c r="C221" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D221" s="8" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="E221" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="7" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" s="7" t="inlineStr">
+        <is>
+          <t>Lacca Forte 400 ml</t>
+        </is>
+      </c>
+      <c r="C222" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D222" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="E222" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="7" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" s="7" t="inlineStr">
+        <is>
+          <t>Lacca Extra Forte 400 ml</t>
+        </is>
+      </c>
+      <c r="C223" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D223" s="8" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="E223" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="7" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" s="7" t="inlineStr">
+        <is>
+          <t>Eco Lacca Invisibile 250 ml</t>
+        </is>
+      </c>
+      <c r="C224" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D224" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="E224" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="7" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" s="7" t="inlineStr">
+        <is>
+          <t>Spray Lucidante 200 ml</t>
+        </is>
+      </c>
+      <c r="C225" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D225" s="8" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="E225" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8044,7 +10459,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Scegli una voce dal menu, oppure aggiungila prima nel foglio Listino." type="list">
-      <formula1>=Listino!$B$2:$B$110</formula1>
+      <formula1>=Listino!$B$2:$B$225</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Contanti,Carta,Satispay,Altro"</formula1>

</xml_diff>

<commit_message>
Completa il listino prodotti: 242 voci
Ultimo blocco: styling More Inside (mousse, cere, dry wax), linea
solari SU, Liquid Spell, Hair Refresher, Hand Sanitizer e Authentic
Formulas. Prezzi corretti a penna confermati dal negozio.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HaLJpnaiiT1t5t7Nsc7fzN
</commit_message>
<xml_diff>
--- a/registro_giornaliero.xlsx
+++ b/registro_giornaliero.xlsx
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E225"/>
+  <dimension ref="A1:E251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5361,6 +5361,552 @@
         <v>31.8</v>
       </c>
       <c r="E225" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="7" t="n">
+        <v>225</v>
+      </c>
+      <c r="B226" s="7" t="inlineStr">
+        <is>
+          <t>Mousse Volume 250 ml</t>
+        </is>
+      </c>
+      <c r="C226" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D226" s="8" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="E226" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="7" t="n">
+        <v>226</v>
+      </c>
+      <c r="B227" s="7" t="inlineStr">
+        <is>
+          <t>Mousse Idratante Ricci 250 ml</t>
+        </is>
+      </c>
+      <c r="C227" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D227" s="8" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="E227" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="7" t="n">
+        <v>227</v>
+      </c>
+      <c r="B228" s="7" t="inlineStr">
+        <is>
+          <t>Spray Texturizzante Secco 250 ml</t>
+        </is>
+      </c>
+      <c r="C228" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D228" s="8" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="E228" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="7" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" s="7" t="inlineStr">
+        <is>
+          <t>Shampoo Secco Invisibile 250 ml</t>
+        </is>
+      </c>
+      <c r="C229" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D229" s="8" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="E229" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="7" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" s="7" t="inlineStr">
+        <is>
+          <t>Cera Illuminante 75 ml</t>
+        </is>
+      </c>
+      <c r="C230" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D230" s="8" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="E230" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="7" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" s="7" t="inlineStr">
+        <is>
+          <t>Pomade per Plasmare 75 ml</t>
+        </is>
+      </c>
+      <c r="C231" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D231" s="8" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="E231" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="7" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" s="7" t="inlineStr">
+        <is>
+          <t>Gomma Texturizzante Media 75 ml</t>
+        </is>
+      </c>
+      <c r="C232" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D232" s="8" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="E232" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="7" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" s="7" t="inlineStr">
+        <is>
+          <t>Argilla Modellante Forte 75 ml</t>
+        </is>
+      </c>
+      <c r="C233" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D233" s="8" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="E233" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="7" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" s="7" t="inlineStr">
+        <is>
+          <t>Cera Forte Asciutta 75 ml</t>
+        </is>
+      </c>
+      <c r="C234" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D234" s="8" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="E234" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="7" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" s="7" t="inlineStr">
+        <is>
+          <t>Dry Wax 200 ml</t>
+        </is>
+      </c>
+      <c r="C235" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - More Inside</t>
+        </is>
+      </c>
+      <c r="D235" s="8" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="E235" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="7" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" s="7" t="inlineStr">
+        <is>
+          <t>SU/Hair &amp; Body Wash 75 ml</t>
+        </is>
+      </c>
+      <c r="C236" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - SU</t>
+        </is>
+      </c>
+      <c r="D236" s="8" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E236" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="7" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" s="7" t="inlineStr">
+        <is>
+          <t>SU/Hair &amp; Body Wash 500 ml</t>
+        </is>
+      </c>
+      <c r="C237" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - SU</t>
+        </is>
+      </c>
+      <c r="D237" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="E237" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="7" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" s="7" t="inlineStr">
+        <is>
+          <t>SU/Hair Mask 150 ml</t>
+        </is>
+      </c>
+      <c r="C238" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - SU</t>
+        </is>
+      </c>
+      <c r="D238" s="8" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="E238" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="7" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" s="7" t="inlineStr">
+        <is>
+          <t>SU/Hair Milk 50 ml</t>
+        </is>
+      </c>
+      <c r="C239" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - SU</t>
+        </is>
+      </c>
+      <c r="D239" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="E239" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="7" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" s="7" t="inlineStr">
+        <is>
+          <t>SU/Hair Milk 135 ml</t>
+        </is>
+      </c>
+      <c r="C240" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - SU</t>
+        </is>
+      </c>
+      <c r="D240" s="8" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="E240" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" s="7" t="inlineStr">
+        <is>
+          <t>SU/Tan Maximizer 150 ml</t>
+        </is>
+      </c>
+      <c r="C241" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - SU</t>
+        </is>
+      </c>
+      <c r="D241" s="8" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="E241" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="7" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" s="7" t="inlineStr">
+        <is>
+          <t>SU/Aftersun 150 ml</t>
+        </is>
+      </c>
+      <c r="C242" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - SU</t>
+        </is>
+      </c>
+      <c r="D242" s="8" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="E242" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="7" t="n">
+        <v>242</v>
+      </c>
+      <c r="B243" s="7" t="inlineStr">
+        <is>
+          <t>SU/Conscious Sunscreen SPF 30 100 ml</t>
+        </is>
+      </c>
+      <c r="C243" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - SU</t>
+        </is>
+      </c>
+      <c r="D243" s="8" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="E243" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="7" t="n">
+        <v>243</v>
+      </c>
+      <c r="B244" s="7" t="inlineStr">
+        <is>
+          <t>Reinforcing Bodifying Fluid 50 ml</t>
+        </is>
+      </c>
+      <c r="C244" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Liquid Spell</t>
+        </is>
+      </c>
+      <c r="D244" s="8" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="E244" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="7" t="n">
+        <v>244</v>
+      </c>
+      <c r="B245" s="7" t="inlineStr">
+        <is>
+          <t>Reinforcing Bodifying Fluid 125 ml</t>
+        </is>
+      </c>
+      <c r="C245" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Liquid Spell</t>
+        </is>
+      </c>
+      <c r="D245" s="8" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="E245" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="7" t="n">
+        <v>245</v>
+      </c>
+      <c r="B246" s="7" t="inlineStr">
+        <is>
+          <t>Hair Refresher - Shampoo a Secco 150 ml</t>
+        </is>
+      </c>
+      <c r="C246" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Hair Refresher</t>
+        </is>
+      </c>
+      <c r="D246" s="8" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="E246" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="7" t="n">
+        <v>246</v>
+      </c>
+      <c r="B247" s="7" t="inlineStr">
+        <is>
+          <t>Hand Sanitizer 75 ml</t>
+        </is>
+      </c>
+      <c r="C247" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Gel del Buon Auspicio</t>
+        </is>
+      </c>
+      <c r="D247" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E247" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="7" t="n">
+        <v>247</v>
+      </c>
+      <c r="B248" s="7" t="inlineStr">
+        <is>
+          <t>Nettare Lavante 280 ml</t>
+        </is>
+      </c>
+      <c r="C248" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Authentic Formulas</t>
+        </is>
+      </c>
+      <c r="D248" s="8" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="E248" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="7" t="n">
+        <v>248</v>
+      </c>
+      <c r="B249" s="7" t="inlineStr">
+        <is>
+          <t>Balsamo Idratante 150 ml</t>
+        </is>
+      </c>
+      <c r="C249" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Authentic Formulas</t>
+        </is>
+      </c>
+      <c r="D249" s="8" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="E249" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="7" t="n">
+        <v>249</v>
+      </c>
+      <c r="B250" s="7" t="inlineStr">
+        <is>
+          <t>Burro Restitutivo 200 ml</t>
+        </is>
+      </c>
+      <c r="C250" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Authentic Formulas</t>
+        </is>
+      </c>
+      <c r="D250" s="8" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="E250" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="B251" s="7" t="inlineStr">
+        <is>
+          <t>Olio Nutriente 140 ml</t>
+        </is>
+      </c>
+      <c r="C251" s="7" t="inlineStr">
+        <is>
+          <t>Prodotto - Authentic Formulas</t>
+        </is>
+      </c>
+      <c r="D251" s="8" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="E251" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10459,7 +11005,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Scegli una voce dal menu, oppure aggiungila prima nel foglio Listino." type="list">
-      <formula1>=Listino!$B$2:$B$225</formula1>
+      <formula1>=Listino!$B$2:$B$251</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Contanti,Carta,Satispay,Altro"</formula1>

</xml_diff>

<commit_message>
Aggiungi la scheda Pieghe del gestionale (6 servizi)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HaLJpnaiiT1t5t7Nsc7fzN
</commit_message>
<xml_diff>
--- a/registro_giornaliero.xlsx
+++ b/registro_giornaliero.xlsx
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E299"/>
+  <dimension ref="A1:E305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1730,18 +1730,18 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Shampoo Argento 280 ml</t>
+          <t>Piega Capello Corto</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Alchemic</t>
+          <t>Servizio - Pieghe</t>
         </is>
       </c>
       <c r="D58" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="E58" s="5" t="n"/>
+        <v>18</v>
+      </c>
+      <c r="E58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n">
@@ -1749,18 +1749,18 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Conditioner Argento 250 ml</t>
+          <t>Piega Capello Lungo da</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Alchemic</t>
+          <t>Servizio - Pieghe</t>
         </is>
       </c>
       <c r="D59" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="E59" s="5" t="n"/>
+        <v>19</v>
+      </c>
+      <c r="E59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
@@ -1768,18 +1768,18 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Shampoo Cioccolato 280 ml</t>
+          <t>Piega Elab da</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Alchemic</t>
+          <t>Servizio - Pieghe</t>
         </is>
       </c>
       <c r="D60" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="E60" s="5" t="n"/>
+        <v>20</v>
+      </c>
+      <c r="E60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n">
@@ -1787,18 +1787,18 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Conditioner Cioccolato 250 ml</t>
+          <t>Acconciatura da</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Alchemic</t>
+          <t>Servizio - Pieghe</t>
         </is>
       </c>
       <c r="D61" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="E61" s="5" t="n"/>
+        <v>30</v>
+      </c>
+      <c r="E61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n">
@@ -1806,18 +1806,18 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Shampoo Dorato 280 ml</t>
+          <t>Acconciatura Sposa da</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Alchemic</t>
+          <t>Servizio - Pieghe</t>
         </is>
       </c>
       <c r="D62" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="E62" s="5" t="n"/>
+        <v>130</v>
+      </c>
+      <c r="E62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n">
@@ -1825,18 +1825,18 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Conditioner Dorato 250 ml</t>
+          <t>Treccine da</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Alchemic</t>
+          <t>Servizio - Pieghe</t>
         </is>
       </c>
       <c r="D63" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="E63" s="5" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="E63" s="7" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Shampoo Rosso 280 ml</t>
+          <t>Shampoo Argento 280 ml</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Conditioner Rosso 250 ml</t>
+          <t>Conditioner Argento 250 ml</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Shampoo Tabacco 280 ml</t>
+          <t>Shampoo Cioccolato 280 ml</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Conditioner Tabacco 250 ml</t>
+          <t>Conditioner Cioccolato 250 ml</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Shampoo Ramato 280 ml</t>
+          <t>Shampoo Dorato 280 ml</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Conditioner Ramato 250 ml</t>
+          <t>Conditioner Dorato 250 ml</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
@@ -1958,16 +1958,16 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Conditioner Rosa 250 ml</t>
+          <t>Shampoo Rosso 280 ml</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Creative Conditioner</t>
+          <t>Prodotto - Alchemic</t>
         </is>
       </c>
       <c r="D70" s="6" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="E70" s="5" t="n"/>
     </row>
@@ -1977,12 +1977,12 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>Conditioner Blu Marino 250 ml</t>
+          <t>Conditioner Rosso 250 ml</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Creative Conditioner</t>
+          <t>Prodotto - Alchemic</t>
         </is>
       </c>
       <c r="D71" s="6" t="n">
@@ -1996,16 +1996,16 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Conditioner Blu Ottanio 250 ml</t>
+          <t>Shampoo Tabacco 280 ml</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Creative Conditioner</t>
+          <t>Prodotto - Alchemic</t>
         </is>
       </c>
       <c r="D72" s="6" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="E72" s="5" t="n"/>
     </row>
@@ -2015,12 +2015,12 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>Conditioner Corallo 250 ml</t>
+          <t>Conditioner Tabacco 250 ml</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Creative Conditioner</t>
+          <t>Prodotto - Alchemic</t>
         </is>
       </c>
       <c r="D73" s="6" t="n">
@@ -2034,16 +2034,16 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>MINU/ Shampoo 75 ml</t>
+          <t>Shampoo Ramato 280 ml</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Essential Haircare</t>
+          <t>Prodotto - Alchemic</t>
         </is>
       </c>
       <c r="D74" s="6" t="n">
-        <v>9.4</v>
+        <v>22</v>
       </c>
       <c r="E74" s="5" t="n"/>
     </row>
@@ -2053,16 +2053,16 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>MINU/ Shampoo 250 ml</t>
+          <t>Conditioner Ramato 250 ml</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Essential Haircare</t>
+          <t>Prodotto - Alchemic</t>
         </is>
       </c>
       <c r="D75" s="6" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E75" s="5" t="n"/>
     </row>
@@ -2072,16 +2072,16 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>MINU/ Shampoo 1000 ml</t>
+          <t>Conditioner Rosa 250 ml</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Essential Haircare</t>
+          <t>Prodotto - Creative Conditioner</t>
         </is>
       </c>
       <c r="D76" s="6" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="E76" s="5" t="n"/>
     </row>
@@ -2091,16 +2091,16 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>MINU/ Conditioner 75 ml</t>
+          <t>Conditioner Blu Marino 250 ml</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Essential Haircare</t>
+          <t>Prodotto - Creative Conditioner</t>
         </is>
       </c>
       <c r="D77" s="6" t="n">
-        <v>9.800000000000001</v>
+        <v>35</v>
       </c>
       <c r="E77" s="5" t="n"/>
     </row>
@@ -2110,16 +2110,16 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>MINU/ Conditioner 250 ml</t>
+          <t>Conditioner Blu Ottanio 250 ml</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Essential Haircare</t>
+          <t>Prodotto - Creative Conditioner</t>
         </is>
       </c>
       <c r="D78" s="6" t="n">
-        <v>23.8</v>
+        <v>35</v>
       </c>
       <c r="E78" s="5" t="n"/>
     </row>
@@ -2129,16 +2129,16 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>MINU/ Conditioner 1000 ml</t>
+          <t>Conditioner Corallo 250 ml</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Essential Haircare</t>
+          <t>Prodotto - Creative Conditioner</t>
         </is>
       </c>
       <c r="D79" s="6" t="n">
-        <v>71.40000000000001</v>
+        <v>35</v>
       </c>
       <c r="E79" s="5" t="n"/>
     </row>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>MINU/ Hair Mask 75 ml</t>
+          <t>MINU/ Shampoo 75 ml</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
@@ -2157,7 +2157,7 @@
         </is>
       </c>
       <c r="D80" s="6" t="n">
-        <v>10</v>
+        <v>9.4</v>
       </c>
       <c r="E80" s="5" t="n"/>
     </row>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>MINU/ Hair Mask 250 ml</t>
+          <t>MINU/ Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
@@ -2176,7 +2176,7 @@
         </is>
       </c>
       <c r="D81" s="6" t="n">
-        <v>27.6</v>
+        <v>20</v>
       </c>
       <c r="E81" s="5" t="n"/>
     </row>
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>MINU/ Hair Mask 1000 ml</t>
+          <t>MINU/ Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
@@ -2195,7 +2195,7 @@
         </is>
       </c>
       <c r="D82" s="6" t="n">
-        <v>82.8</v>
+        <v>60</v>
       </c>
       <c r="E82" s="5" t="n"/>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>MINU/ Hair Serum 150 ml</t>
+          <t>MINU/ Conditioner 75 ml</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
@@ -2214,7 +2214,7 @@
         </is>
       </c>
       <c r="D83" s="6" t="n">
-        <v>23.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E83" s="5" t="n"/>
     </row>
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>NOUNOU/ Shampoo 75 ml</t>
+          <t>MINU/ Conditioner 250 ml</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="D84" s="6" t="n">
-        <v>9.4</v>
+        <v>23.8</v>
       </c>
       <c r="E84" s="5" t="n"/>
     </row>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>NOUNOU/ Shampoo 250 ml</t>
+          <t>MINU/ Conditioner 1000 ml</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
@@ -2252,7 +2252,7 @@
         </is>
       </c>
       <c r="D85" s="6" t="n">
-        <v>20</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="E85" s="5" t="n"/>
     </row>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>NOUNOU/ Shampoo 1000 ml</t>
+          <t>MINU/ Hair Mask 75 ml</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="D86" s="6" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="E86" s="5" t="n"/>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>NOUNOU/ Conditioner 75 ml</t>
+          <t>MINU/ Hair Mask 250 ml</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
@@ -2290,7 +2290,7 @@
         </is>
       </c>
       <c r="D87" s="6" t="n">
-        <v>9.800000000000001</v>
+        <v>27.6</v>
       </c>
       <c r="E87" s="5" t="n"/>
     </row>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>NOUNOU/ Conditioner 250 ml</t>
+          <t>MINU/ Hair Mask 1000 ml</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="D88" s="6" t="n">
-        <v>23.8</v>
+        <v>82.8</v>
       </c>
       <c r="E88" s="5" t="n"/>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>NOUNOU/ Conditioner 1000 ml</t>
+          <t>MINU/ Hair Serum 150 ml</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
@@ -2328,7 +2328,7 @@
         </is>
       </c>
       <c r="D89" s="6" t="n">
-        <v>71.40000000000001</v>
+        <v>23.9</v>
       </c>
       <c r="E89" s="5" t="n"/>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>NOUNOU/ Hair Mask 75 ml</t>
+          <t>NOUNOU/ Shampoo 75 ml</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="D90" s="6" t="n">
-        <v>10</v>
+        <v>9.4</v>
       </c>
       <c r="E90" s="5" t="n"/>
     </row>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>NOUNOU/ Hair Mask 250 ml</t>
+          <t>NOUNOU/ Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
@@ -2366,7 +2366,7 @@
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>27.6</v>
+        <v>20</v>
       </c>
       <c r="E91" s="5" t="n"/>
     </row>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>NOUNOU/ Hair Mask 1000 ml</t>
+          <t>NOUNOU/ Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
@@ -2385,7 +2385,7 @@
         </is>
       </c>
       <c r="D92" s="6" t="n">
-        <v>82.8</v>
+        <v>60</v>
       </c>
       <c r="E92" s="5" t="n"/>
     </row>
@@ -2395,7 +2395,7 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>MELU/ Shampoo 75 ml</t>
+          <t>NOUNOU/ Conditioner 75 ml</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>9.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E93" s="5" t="n"/>
     </row>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>MELU/ Shampoo 250 ml</t>
+          <t>NOUNOU/ Conditioner 250 ml</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="D94" s="6" t="n">
-        <v>20</v>
+        <v>23.8</v>
       </c>
       <c r="E94" s="5" t="n"/>
     </row>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>MELU/ Shampoo 1000 ml</t>
+          <t>NOUNOU/ Conditioner 1000 ml</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
@@ -2442,7 +2442,7 @@
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>60</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="E95" s="5" t="n"/>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>MELU/ Conditioner 75 ml</t>
+          <t>NOUNOU/ Hair Mask 75 ml</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
@@ -2461,7 +2461,7 @@
         </is>
       </c>
       <c r="D96" s="6" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="E96" s="5" t="n"/>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>MELU/ Conditioner 250 ml</t>
+          <t>NOUNOU/ Hair Mask 250 ml</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
@@ -2480,7 +2480,7 @@
         </is>
       </c>
       <c r="D97" s="6" t="n">
-        <v>23.8</v>
+        <v>27.6</v>
       </c>
       <c r="E97" s="5" t="n"/>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>MELU/ Conditioner 1000 ml</t>
+          <t>NOUNOU/ Hair Mask 1000 ml</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
@@ -2499,7 +2499,7 @@
         </is>
       </c>
       <c r="D98" s="6" t="n">
-        <v>71.40000000000001</v>
+        <v>82.8</v>
       </c>
       <c r="E98" s="5" t="n"/>
     </row>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>MELU/ Hair Shield 250 ml</t>
+          <t>MELU/ Shampoo 75 ml</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
@@ -2518,7 +2518,7 @@
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>34.6</v>
+        <v>9.4</v>
       </c>
       <c r="E99" s="5" t="n"/>
     </row>
@@ -2528,7 +2528,7 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>DEDE/ Shampoo 75 ml</t>
+          <t>MELU/ Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D100" s="6" t="n">
-        <v>9.4</v>
+        <v>20</v>
       </c>
       <c r="E100" s="5" t="n"/>
     </row>
@@ -2547,7 +2547,7 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>DEDE/ Shampoo 250 ml</t>
+          <t>MELU/ Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
@@ -2556,7 +2556,7 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E101" s="5" t="n"/>
     </row>
@@ -2566,7 +2566,7 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>DEDE/ Shampoo 1000 ml</t>
+          <t>MELU/ Conditioner 75 ml</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
@@ -2575,7 +2575,7 @@
         </is>
       </c>
       <c r="D102" s="6" t="n">
-        <v>60</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E102" s="5" t="n"/>
     </row>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>DEDE/ Conditioner 75 ml</t>
+          <t>MELU/ Conditioner 250 ml</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
@@ -2594,7 +2594,7 @@
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>9.800000000000001</v>
+        <v>23.8</v>
       </c>
       <c r="E103" s="5" t="n"/>
     </row>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>DEDE/ Conditioner 250 ml</t>
+          <t>MELU/ Conditioner 1000 ml</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
@@ -2613,7 +2613,7 @@
         </is>
       </c>
       <c r="D104" s="6" t="n">
-        <v>23.8</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="E104" s="5" t="n"/>
     </row>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>DEDE/ Conditioner 1000 ml</t>
+          <t>MELU/ Hair Shield 250 ml</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
@@ -2632,7 +2632,7 @@
         </is>
       </c>
       <c r="D105" s="6" t="n">
-        <v>71.40000000000001</v>
+        <v>34.6</v>
       </c>
       <c r="E105" s="5" t="n"/>
     </row>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>DEDE/ Hair Mist 250 ml</t>
+          <t>DEDE/ Shampoo 75 ml</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="D106" s="6" t="n">
-        <v>29</v>
+        <v>9.4</v>
       </c>
       <c r="E106" s="5" t="n"/>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>VOLU/ Shampoo 75 ml</t>
+          <t>DEDE/ Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="D107" s="6" t="n">
-        <v>9.4</v>
+        <v>20</v>
       </c>
       <c r="E107" s="5" t="n"/>
     </row>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>VOLU/ Shampoo 250 ml</t>
+          <t>DEDE/ Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
@@ -2689,7 +2689,7 @@
         </is>
       </c>
       <c r="D108" s="6" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E108" s="5" t="n"/>
     </row>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>VOLU/ Shampoo 1000 ml</t>
+          <t>DEDE/ Conditioner 75 ml</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
@@ -2708,7 +2708,7 @@
         </is>
       </c>
       <c r="D109" s="6" t="n">
-        <v>60</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E109" s="5" t="n"/>
     </row>
@@ -2718,7 +2718,7 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>VOLU/ Hair Mist 250 ml</t>
+          <t>DEDE/ Conditioner 250 ml</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
@@ -2727,7 +2727,7 @@
         </is>
       </c>
       <c r="D110" s="6" t="n">
-        <v>34.6</v>
+        <v>23.8</v>
       </c>
       <c r="E110" s="5" t="n"/>
     </row>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>SOLU/ Shampoo 75 ml</t>
+          <t>DEDE/ Conditioner 1000 ml</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="D111" s="6" t="n">
-        <v>9.4</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="E111" s="5" t="n"/>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>SOLU/ Shampoo 250 ml</t>
+          <t>DEDE/ Hair Mist 250 ml</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
@@ -2765,7 +2765,7 @@
         </is>
       </c>
       <c r="D112" s="6" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E112" s="5" t="n"/>
     </row>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>SOLU/ Shampoo 1000 ml</t>
+          <t>VOLU/ Shampoo 75 ml</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
@@ -2784,7 +2784,7 @@
         </is>
       </c>
       <c r="D113" s="6" t="n">
-        <v>60</v>
+        <v>9.4</v>
       </c>
       <c r="E113" s="5" t="n"/>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>SOLU/ Sea Salt Scrub Cleanser 75 ml</t>
+          <t>VOLU/ Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
@@ -2803,7 +2803,7 @@
         </is>
       </c>
       <c r="D114" s="6" t="n">
-        <v>11.6</v>
+        <v>20</v>
       </c>
       <c r="E114" s="5" t="n"/>
     </row>
@@ -2813,7 +2813,7 @@
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>SOLU/ Sea Salt Scrub Cleanser 250 ml</t>
+          <t>VOLU/ Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
@@ -2822,7 +2822,7 @@
         </is>
       </c>
       <c r="D115" s="6" t="n">
-        <v>28.6</v>
+        <v>60</v>
       </c>
       <c r="E115" s="5" t="n"/>
     </row>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>MOMO/ Shampoo 75 ml</t>
+          <t>VOLU/ Hair Mist 250 ml</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="D116" s="6" t="n">
-        <v>9.4</v>
+        <v>34.6</v>
       </c>
       <c r="E116" s="5" t="n"/>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>MOMO/ Shampoo 250 ml</t>
+          <t>SOLU/ Shampoo 75 ml</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
@@ -2860,7 +2860,7 @@
         </is>
       </c>
       <c r="D117" s="6" t="n">
-        <v>20</v>
+        <v>9.4</v>
       </c>
       <c r="E117" s="5" t="n"/>
     </row>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>MOMO/ Shampoo 1000 ml</t>
+          <t>SOLU/ Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="D118" s="6" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E118" s="5" t="n"/>
     </row>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="B119" s="5" t="inlineStr">
         <is>
-          <t>MOMO/ Conditioner 75 ml</t>
+          <t>SOLU/ Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
@@ -2898,7 +2898,7 @@
         </is>
       </c>
       <c r="D119" s="6" t="n">
-        <v>9.800000000000001</v>
+        <v>60</v>
       </c>
       <c r="E119" s="5" t="n"/>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>MOMO/ Conditioner 250 ml</t>
+          <t>SOLU/ Sea Salt Scrub Cleanser 75 ml</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
@@ -2917,7 +2917,7 @@
         </is>
       </c>
       <c r="D120" s="6" t="n">
-        <v>23.8</v>
+        <v>11.6</v>
       </c>
       <c r="E120" s="5" t="n"/>
     </row>
@@ -2927,7 +2927,7 @@
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>MOMO/ Conditioner 1000 ml</t>
+          <t>SOLU/ Sea Salt Scrub Cleanser 250 ml</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
@@ -2936,7 +2936,7 @@
         </is>
       </c>
       <c r="D121" s="6" t="n">
-        <v>71.40000000000001</v>
+        <v>28.6</v>
       </c>
       <c r="E121" s="5" t="n"/>
     </row>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>MOMO/ Hair Potion 150 ml</t>
+          <t>MOMO/ Shampoo 75 ml</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
@@ -2955,7 +2955,7 @@
         </is>
       </c>
       <c r="D122" s="6" t="n">
-        <v>23.5</v>
+        <v>9.4</v>
       </c>
       <c r="E122" s="5" t="n"/>
     </row>
@@ -2965,7 +2965,7 @@
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Cleansing Cream 500 ml</t>
+          <t>MOMO/ Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
@@ -2974,7 +2974,7 @@
         </is>
       </c>
       <c r="D123" s="6" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E123" s="5" t="n"/>
     </row>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Shampoo 75 ml</t>
+          <t>MOMO/ Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C124" s="5" t="inlineStr">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="D124" s="6" t="n">
-        <v>9.4</v>
+        <v>60</v>
       </c>
       <c r="E124" s="5" t="n"/>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="B125" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Shampoo 250 ml</t>
+          <t>MOMO/ Conditioner 75 ml</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="D125" s="6" t="n">
-        <v>20</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E125" s="5" t="n"/>
     </row>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Shampoo 1000 ml</t>
+          <t>MOMO/ Conditioner 250 ml</t>
         </is>
       </c>
       <c r="C126" s="5" t="inlineStr">
@@ -3031,7 +3031,7 @@
         </is>
       </c>
       <c r="D126" s="6" t="n">
-        <v>60</v>
+        <v>23.8</v>
       </c>
       <c r="E126" s="5" t="n"/>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Conditioner 75 ml</t>
+          <t>MOMO/ Conditioner 1000 ml</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
@@ -3050,7 +3050,7 @@
         </is>
       </c>
       <c r="D127" s="6" t="n">
-        <v>9.800000000000001</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="E127" s="5" t="n"/>
     </row>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Conditioner 250 ml</t>
+          <t>MOMO/ Hair Potion 150 ml</t>
         </is>
       </c>
       <c r="C128" s="5" t="inlineStr">
@@ -3069,7 +3069,7 @@
         </is>
       </c>
       <c r="D128" s="6" t="n">
-        <v>23.8</v>
+        <v>23.5</v>
       </c>
       <c r="E128" s="5" t="n"/>
     </row>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Conditioner 1000 ml</t>
+          <t>LOVE/ Curl Cleansing Cream 500 ml</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
@@ -3088,7 +3088,7 @@
         </is>
       </c>
       <c r="D129" s="6" t="n">
-        <v>71.40000000000001</v>
+        <v>36</v>
       </c>
       <c r="E129" s="5" t="n"/>
     </row>
@@ -3098,7 +3098,7 @@
       </c>
       <c r="B130" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Mask 75 ml</t>
+          <t>LOVE/ Curl Shampoo 75 ml</t>
         </is>
       </c>
       <c r="C130" s="5" t="inlineStr">
@@ -3107,7 +3107,7 @@
         </is>
       </c>
       <c r="D130" s="6" t="n">
-        <v>10</v>
+        <v>9.4</v>
       </c>
       <c r="E130" s="5" t="n"/>
     </row>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="B131" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Mask 250 ml</t>
+          <t>LOVE/ Curl Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
@@ -3126,7 +3126,7 @@
         </is>
       </c>
       <c r="D131" s="6" t="n">
-        <v>27.6</v>
+        <v>20</v>
       </c>
       <c r="E131" s="5" t="n"/>
     </row>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="B132" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Mask 1000 ml</t>
+          <t>LOVE/ Curl Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="D132" s="6" t="n">
-        <v>82.8</v>
+        <v>60</v>
       </c>
       <c r="E132" s="5" t="n"/>
     </row>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Primer 150 ml</t>
+          <t>LOVE/ Curl Conditioner 75 ml</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
@@ -3164,7 +3164,7 @@
         </is>
       </c>
       <c r="D133" s="6" t="n">
-        <v>25.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E133" s="5" t="n"/>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Cream 150 ml</t>
+          <t>LOVE/ Curl Conditioner 250 ml</t>
         </is>
       </c>
       <c r="C134" s="5" t="inlineStr">
@@ -3183,7 +3183,7 @@
         </is>
       </c>
       <c r="D134" s="6" t="n">
-        <v>25.6</v>
+        <v>23.8</v>
       </c>
       <c r="E134" s="5" t="n"/>
     </row>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="B135" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Controller 150 ml</t>
+          <t>LOVE/ Curl Conditioner 1000 ml</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
@@ -3202,7 +3202,7 @@
         </is>
       </c>
       <c r="D135" s="6" t="n">
-        <v>25.6</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="E135" s="5" t="n"/>
     </row>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="B136" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Revitalizer 75 ml</t>
+          <t>LOVE/ Curl Mask 75 ml</t>
         </is>
       </c>
       <c r="C136" s="5" t="inlineStr">
@@ -3221,7 +3221,7 @@
         </is>
       </c>
       <c r="D136" s="6" t="n">
-        <v>11.2</v>
+        <v>10</v>
       </c>
       <c r="E136" s="5" t="n"/>
     </row>
@@ -3231,7 +3231,7 @@
       </c>
       <c r="B137" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Curl Revitalizer 250 ml</t>
+          <t>LOVE/ Curl Mask 250 ml</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
@@ -3240,7 +3240,7 @@
         </is>
       </c>
       <c r="D137" s="6" t="n">
-        <v>30.8</v>
+        <v>27.6</v>
       </c>
       <c r="E137" s="5" t="n"/>
     </row>
@@ -3250,7 +3250,7 @@
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Shampoo (Smoothing) 75 ml</t>
+          <t>LOVE/ Curl Mask 1000 ml</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="D138" s="6" t="n">
-        <v>9.4</v>
+        <v>82.8</v>
       </c>
       <c r="E138" s="5" t="n"/>
     </row>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Shampoo (Smoothing) 250 ml</t>
+          <t>LOVE/ Curl Primer 150 ml</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
@@ -3278,7 +3278,7 @@
         </is>
       </c>
       <c r="D139" s="6" t="n">
-        <v>20</v>
+        <v>25.6</v>
       </c>
       <c r="E139" s="5" t="n"/>
     </row>
@@ -3288,7 +3288,7 @@
       </c>
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Shampoo (Smoothing) 1000 ml</t>
+          <t>LOVE/ Curl Cream 150 ml</t>
         </is>
       </c>
       <c r="C140" s="5" t="inlineStr">
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="D140" s="6" t="n">
-        <v>60</v>
+        <v>25.6</v>
       </c>
       <c r="E140" s="5" t="n"/>
     </row>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="B141" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Conditioner (Smoothing) 75 ml</t>
+          <t>LOVE/ Curl Controller 150 ml</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
@@ -3316,7 +3316,7 @@
         </is>
       </c>
       <c r="D141" s="6" t="n">
-        <v>9.800000000000001</v>
+        <v>25.6</v>
       </c>
       <c r="E141" s="5" t="n"/>
     </row>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="B142" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Conditioner (Smoothing) 250 ml</t>
+          <t>LOVE/ Curl Revitalizer 75 ml</t>
         </is>
       </c>
       <c r="C142" s="5" t="inlineStr">
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="D142" s="6" t="n">
-        <v>23.8</v>
+        <v>11.2</v>
       </c>
       <c r="E142" s="5" t="n"/>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="B143" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Conditioner (Smoothing) 1000 ml</t>
+          <t>LOVE/ Curl Revitalizer 250 ml</t>
         </is>
       </c>
       <c r="C143" s="5" t="inlineStr">
@@ -3354,7 +3354,7 @@
         </is>
       </c>
       <c r="D143" s="6" t="n">
-        <v>71.40000000000001</v>
+        <v>30.8</v>
       </c>
       <c r="E143" s="5" t="n"/>
     </row>
@@ -3364,7 +3364,7 @@
       </c>
       <c r="B144" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Instant Mask 75 ml</t>
+          <t>LOVE/ Shampoo (Smoothing) 75 ml</t>
         </is>
       </c>
       <c r="C144" s="5" t="inlineStr">
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="D144" s="6" t="n">
-        <v>10</v>
+        <v>9.4</v>
       </c>
       <c r="E144" s="5" t="n"/>
     </row>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B145" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Instant Mask 250 ml</t>
+          <t>LOVE/ Shampoo (Smoothing) 250 ml</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr">
@@ -3392,7 +3392,7 @@
         </is>
       </c>
       <c r="D145" s="6" t="n">
-        <v>27.6</v>
+        <v>20</v>
       </c>
       <c r="E145" s="5" t="n"/>
     </row>
@@ -3402,7 +3402,7 @@
       </c>
       <c r="B146" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Instant Mask 1000 ml</t>
+          <t>LOVE/ Shampoo (Smoothing) 1000 ml</t>
         </is>
       </c>
       <c r="C146" s="5" t="inlineStr">
@@ -3411,7 +3411,7 @@
         </is>
       </c>
       <c r="D146" s="6" t="n">
-        <v>82.8</v>
+        <v>60</v>
       </c>
       <c r="E146" s="5" t="n"/>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="B147" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Hair Smoother 150 ml</t>
+          <t>LOVE/ Conditioner (Smoothing) 75 ml</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr">
@@ -3430,7 +3430,7 @@
         </is>
       </c>
       <c r="D147" s="6" t="n">
-        <v>23.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E147" s="5" t="n"/>
     </row>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="B148" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Perfector 150 ml</t>
+          <t>LOVE/ Conditioner (Smoothing) 250 ml</t>
         </is>
       </c>
       <c r="C148" s="5" t="inlineStr">
@@ -3449,7 +3449,7 @@
         </is>
       </c>
       <c r="D148" s="6" t="n">
-        <v>27.6</v>
+        <v>23.8</v>
       </c>
       <c r="E148" s="5" t="n"/>
     </row>
@@ -3459,16 +3459,16 @@
       </c>
       <c r="B149" s="5" t="inlineStr">
         <is>
-          <t>Hair&amp;Body Wash Bar 100 gr</t>
+          <t>LOVE/ Conditioner (Smoothing) 1000 ml</t>
         </is>
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Grow Beautiful</t>
+          <t>Prodotto - Essential Haircare</t>
         </is>
       </c>
       <c r="D149" s="6" t="n">
-        <v>20</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="E149" s="5" t="n"/>
     </row>
@@ -3478,16 +3478,16 @@
       </c>
       <c r="B150" s="5" t="inlineStr">
         <is>
-          <t>MOMO/ Shampoo Bar 100 gr</t>
+          <t>LOVE/ Instant Mask 75 ml</t>
         </is>
       </c>
       <c r="C150" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Shampoo Bar</t>
+          <t>Prodotto - Essential Haircare</t>
         </is>
       </c>
       <c r="D150" s="6" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E150" s="5" t="n"/>
     </row>
@@ -3497,16 +3497,16 @@
       </c>
       <c r="B151" s="5" t="inlineStr">
         <is>
-          <t>DEDE/ Shampoo Bar 100 gr</t>
+          <t>LOVE/ Instant Mask 250 ml</t>
         </is>
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Shampoo Bar</t>
+          <t>Prodotto - Essential Haircare</t>
         </is>
       </c>
       <c r="D151" s="6" t="n">
-        <v>20</v>
+        <v>27.6</v>
       </c>
       <c r="E151" s="5" t="n"/>
     </row>
@@ -3516,16 +3516,16 @@
       </c>
       <c r="B152" s="5" t="inlineStr">
         <is>
-          <t>VOLU/ Shampoo Bar 100 gr</t>
+          <t>LOVE/ Instant Mask 1000 ml</t>
         </is>
       </c>
       <c r="C152" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Shampoo Bar</t>
+          <t>Prodotto - Essential Haircare</t>
         </is>
       </c>
       <c r="D152" s="6" t="n">
-        <v>20</v>
+        <v>82.8</v>
       </c>
       <c r="E152" s="5" t="n"/>
     </row>
@@ -3535,16 +3535,16 @@
       </c>
       <c r="B153" s="5" t="inlineStr">
         <is>
-          <t>LOVE/ Shampoo Bar 100 gr</t>
+          <t>LOVE/ Hair Smoother 150 ml</t>
         </is>
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Shampoo Bar</t>
+          <t>Prodotto - Essential Haircare</t>
         </is>
       </c>
       <c r="D153" s="6" t="n">
-        <v>20</v>
+        <v>23.9</v>
       </c>
       <c r="E153" s="5" t="n"/>
     </row>
@@ -3554,16 +3554,16 @@
       </c>
       <c r="B154" s="5" t="inlineStr">
         <is>
-          <t>The Purity Circle 50 ml</t>
+          <t>LOVE/ Perfector 150 ml</t>
         </is>
       </c>
       <c r="C154" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Circle Chronicles</t>
+          <t>Prodotto - Essential Haircare</t>
         </is>
       </c>
       <c r="D154" s="6" t="n">
-        <v>9.5</v>
+        <v>27.6</v>
       </c>
       <c r="E154" s="5" t="n"/>
     </row>
@@ -3573,16 +3573,16 @@
       </c>
       <c r="B155" s="5" t="inlineStr">
         <is>
-          <t>The Quick Fix Circle 50 ml</t>
+          <t>Hair&amp;Body Wash Bar 100 gr</t>
         </is>
       </c>
       <c r="C155" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Circle Chronicles</t>
+          <t>Prodotto - Grow Beautiful</t>
         </is>
       </c>
       <c r="D155" s="6" t="n">
-        <v>9.5</v>
+        <v>20</v>
       </c>
       <c r="E155" s="5" t="n"/>
     </row>
@@ -3592,16 +3592,16 @@
       </c>
       <c r="B156" s="5" t="inlineStr">
         <is>
-          <t>The Renaissance Circle 50 ml</t>
+          <t>MOMO/ Shampoo Bar 100 gr</t>
         </is>
       </c>
       <c r="C156" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Circle Chronicles</t>
+          <t>Prodotto - Shampoo Bar</t>
         </is>
       </c>
       <c r="D156" s="6" t="n">
-        <v>9.5</v>
+        <v>20</v>
       </c>
       <c r="E156" s="5" t="n"/>
     </row>
@@ -3611,16 +3611,16 @@
       </c>
       <c r="B157" s="5" t="inlineStr">
         <is>
-          <t>The Spotlight Circle 50 ml</t>
+          <t>DEDE/ Shampoo Bar 100 gr</t>
         </is>
       </c>
       <c r="C157" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Circle Chronicles</t>
+          <t>Prodotto - Shampoo Bar</t>
         </is>
       </c>
       <c r="D157" s="6" t="n">
-        <v>9.5</v>
+        <v>20</v>
       </c>
       <c r="E157" s="5" t="n"/>
     </row>
@@ -3630,16 +3630,16 @@
       </c>
       <c r="B158" s="5" t="inlineStr">
         <is>
-          <t>The Wake-Up Circle 50 ml</t>
+          <t>VOLU/ Shampoo Bar 100 gr</t>
         </is>
       </c>
       <c r="C158" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Circle Chronicles</t>
+          <t>Prodotto - Shampoo Bar</t>
         </is>
       </c>
       <c r="D158" s="6" t="n">
-        <v>9.5</v>
+        <v>20</v>
       </c>
       <c r="E158" s="5" t="n"/>
     </row>
@@ -3649,16 +3649,16 @@
       </c>
       <c r="B159" s="5" t="inlineStr">
         <is>
-          <t>The Let It Go Circle 50 ml</t>
+          <t>LOVE/ Shampoo Bar 100 gr</t>
         </is>
       </c>
       <c r="C159" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Circle Chronicles</t>
+          <t>Prodotto - Shampoo Bar</t>
         </is>
       </c>
       <c r="D159" s="6" t="n">
-        <v>9.5</v>
+        <v>20</v>
       </c>
       <c r="E159" s="5" t="n"/>
     </row>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="B160" s="5" t="inlineStr">
         <is>
-          <t>The Restless Circle 50 ml</t>
+          <t>The Purity Circle 50 ml</t>
         </is>
       </c>
       <c r="C160" s="5" t="inlineStr">
@@ -3687,16 +3687,16 @@
       </c>
       <c r="B161" s="5" t="inlineStr">
         <is>
-          <t>Renewing Shampoo 100 ml</t>
+          <t>The Quick Fix Circle 50 ml</t>
         </is>
       </c>
       <c r="C161" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Naturaltech</t>
+          <t>Prodotto - Circle Chronicles</t>
         </is>
       </c>
       <c r="D161" s="6" t="n">
-        <v>13.3</v>
+        <v>9.5</v>
       </c>
       <c r="E161" s="5" t="n"/>
     </row>
@@ -3706,16 +3706,16 @@
       </c>
       <c r="B162" s="5" t="inlineStr">
         <is>
-          <t>Renewing Shampoo 250 ml</t>
+          <t>The Renaissance Circle 50 ml</t>
         </is>
       </c>
       <c r="C162" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Naturaltech</t>
+          <t>Prodotto - Circle Chronicles</t>
         </is>
       </c>
       <c r="D162" s="6" t="n">
-        <v>22.9</v>
+        <v>9.5</v>
       </c>
       <c r="E162" s="5" t="n"/>
     </row>
@@ -3725,16 +3725,16 @@
       </c>
       <c r="B163" s="5" t="inlineStr">
         <is>
-          <t>Renewing Shampoo 1000 ml</t>
+          <t>The Spotlight Circle 50 ml</t>
         </is>
       </c>
       <c r="C163" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Naturaltech</t>
+          <t>Prodotto - Circle Chronicles</t>
         </is>
       </c>
       <c r="D163" s="6" t="n">
-        <v>68.7</v>
+        <v>9.5</v>
       </c>
       <c r="E163" s="5" t="n"/>
     </row>
@@ -3744,16 +3744,16 @@
       </c>
       <c r="B164" s="5" t="inlineStr">
         <is>
-          <t>Renewing Conditioning Treatment 60 ml</t>
+          <t>The Wake-Up Circle 50 ml</t>
         </is>
       </c>
       <c r="C164" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Naturaltech</t>
+          <t>Prodotto - Circle Chronicles</t>
         </is>
       </c>
       <c r="D164" s="6" t="n">
-        <v>13.2</v>
+        <v>9.5</v>
       </c>
       <c r="E164" s="5" t="n"/>
     </row>
@@ -3763,16 +3763,16 @@
       </c>
       <c r="B165" s="5" t="inlineStr">
         <is>
-          <t>Renewing Conditioning Treatment 250 ml</t>
+          <t>The Let It Go Circle 50 ml</t>
         </is>
       </c>
       <c r="C165" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Naturaltech</t>
+          <t>Prodotto - Circle Chronicles</t>
         </is>
       </c>
       <c r="D165" s="6" t="n">
-        <v>29.5</v>
+        <v>9.5</v>
       </c>
       <c r="E165" s="5" t="n"/>
     </row>
@@ -3782,16 +3782,16 @@
       </c>
       <c r="B166" s="5" t="inlineStr">
         <is>
-          <t>Renewing Conditioning Treatment 1000 ml</t>
+          <t>The Restless Circle 50 ml</t>
         </is>
       </c>
       <c r="C166" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Naturaltech</t>
+          <t>Prodotto - Circle Chronicles</t>
         </is>
       </c>
       <c r="D166" s="6" t="n">
-        <v>87</v>
+        <v>9.5</v>
       </c>
       <c r="E166" s="5" t="n"/>
     </row>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="B167" s="5" t="inlineStr">
         <is>
-          <t>Replumping Shampoo 100 ml</t>
+          <t>Renewing Shampoo 100 ml</t>
         </is>
       </c>
       <c r="C167" s="5" t="inlineStr">
@@ -3820,7 +3820,7 @@
       </c>
       <c r="B168" s="5" t="inlineStr">
         <is>
-          <t>Replumping Shampoo 250 ml</t>
+          <t>Renewing Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C168" s="5" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="B169" s="5" t="inlineStr">
         <is>
-          <t>Replumping Shampoo 1000 ml</t>
+          <t>Renewing Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C169" s="5" t="inlineStr">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="B170" s="5" t="inlineStr">
         <is>
-          <t>Replumping Conditioner 60 ml</t>
+          <t>Renewing Conditioning Treatment 60 ml</t>
         </is>
       </c>
       <c r="C170" s="5" t="inlineStr">
@@ -3877,7 +3877,7 @@
       </c>
       <c r="B171" s="5" t="inlineStr">
         <is>
-          <t>Replumping Conditioner 150 ml</t>
+          <t>Renewing Conditioning Treatment 250 ml</t>
         </is>
       </c>
       <c r="C171" s="5" t="inlineStr">
@@ -3886,7 +3886,7 @@
         </is>
       </c>
       <c r="D171" s="6" t="n">
-        <v>22.2</v>
+        <v>29.5</v>
       </c>
       <c r="E171" s="5" t="n"/>
     </row>
@@ -3896,7 +3896,7 @@
       </c>
       <c r="B172" s="5" t="inlineStr">
         <is>
-          <t>Replumping Conditioner 1000 ml</t>
+          <t>Renewing Conditioning Treatment 1000 ml</t>
         </is>
       </c>
       <c r="C172" s="5" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="B173" s="5" t="inlineStr">
         <is>
-          <t>Replumping Hair Filler Superactive 100 ml</t>
+          <t>Replumping Shampoo 100 ml</t>
         </is>
       </c>
       <c r="C173" s="5" t="inlineStr">
@@ -3924,7 +3924,7 @@
         </is>
       </c>
       <c r="D173" s="6" t="n">
-        <v>40.8</v>
+        <v>13.3</v>
       </c>
       <c r="E173" s="5" t="n"/>
     </row>
@@ -3934,7 +3934,7 @@
       </c>
       <c r="B174" s="5" t="inlineStr">
         <is>
-          <t>Energizing Shampoo 100 ml</t>
+          <t>Replumping Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C174" s="5" t="inlineStr">
@@ -3943,7 +3943,7 @@
         </is>
       </c>
       <c r="D174" s="6" t="n">
-        <v>13.3</v>
+        <v>22.9</v>
       </c>
       <c r="E174" s="5" t="n"/>
     </row>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="B175" s="5" t="inlineStr">
         <is>
-          <t>Energizing Shampoo 250 ml</t>
+          <t>Replumping Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C175" s="5" t="inlineStr">
@@ -3962,7 +3962,7 @@
         </is>
       </c>
       <c r="D175" s="6" t="n">
-        <v>23</v>
+        <v>68.7</v>
       </c>
       <c r="E175" s="5" t="n"/>
     </row>
@@ -3972,7 +3972,7 @@
       </c>
       <c r="B176" s="5" t="inlineStr">
         <is>
-          <t>Energizing Shampoo 1000 ml</t>
+          <t>Replumping Conditioner 60 ml</t>
         </is>
       </c>
       <c r="C176" s="5" t="inlineStr">
@@ -3981,7 +3981,7 @@
         </is>
       </c>
       <c r="D176" s="6" t="n">
-        <v>68.7</v>
+        <v>13.2</v>
       </c>
       <c r="E176" s="5" t="n"/>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="B177" s="5" t="inlineStr">
         <is>
-          <t>Energizing Seasonal Superactive 100 ml</t>
+          <t>Replumping Conditioner 150 ml</t>
         </is>
       </c>
       <c r="C177" s="5" t="inlineStr">
@@ -4000,7 +4000,7 @@
         </is>
       </c>
       <c r="D177" s="6" t="n">
-        <v>74</v>
+        <v>22.2</v>
       </c>
       <c r="E177" s="5" t="n"/>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="B178" s="5" t="inlineStr">
         <is>
-          <t>Energizing Seasonal Superactive 12x6 ml</t>
+          <t>Replumping Conditioner 1000 ml</t>
         </is>
       </c>
       <c r="C178" s="5" t="inlineStr">
@@ -4019,7 +4019,7 @@
         </is>
       </c>
       <c r="D178" s="6" t="n">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="E178" s="5" t="n"/>
     </row>
@@ -4029,7 +4029,7 @@
       </c>
       <c r="B179" s="5" t="inlineStr">
         <is>
-          <t>Energizing Superactive Anytime 100 ml</t>
+          <t>Replumping Hair Filler Superactive 100 ml</t>
         </is>
       </c>
       <c r="C179" s="5" t="inlineStr">
@@ -4038,7 +4038,7 @@
         </is>
       </c>
       <c r="D179" s="6" t="n">
-        <v>85</v>
+        <v>40.8</v>
       </c>
       <c r="E179" s="5" t="n"/>
     </row>
@@ -4048,7 +4048,7 @@
       </c>
       <c r="B180" s="5" t="inlineStr">
         <is>
-          <t>Energizing Gel 150 ml</t>
+          <t>Energizing Shampoo 100 ml</t>
         </is>
       </c>
       <c r="C180" s="5" t="inlineStr">
@@ -4057,7 +4057,7 @@
         </is>
       </c>
       <c r="D180" s="6" t="n">
-        <v>37.6</v>
+        <v>13.3</v>
       </c>
       <c r="E180" s="5" t="n"/>
     </row>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="B181" s="5" t="inlineStr">
         <is>
-          <t>Energizing Thickening Tonic 100 ml</t>
+          <t>Energizing Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C181" s="5" t="inlineStr">
@@ -4076,7 +4076,7 @@
         </is>
       </c>
       <c r="D181" s="6" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="E181" s="5" t="n"/>
     </row>
@@ -4086,7 +4086,7 @@
       </c>
       <c r="B182" s="5" t="inlineStr">
         <is>
-          <t>Purifying Shampoo 100 ml</t>
+          <t>Energizing Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C182" s="5" t="inlineStr">
@@ -4095,7 +4095,7 @@
         </is>
       </c>
       <c r="D182" s="6" t="n">
-        <v>13.3</v>
+        <v>68.7</v>
       </c>
       <c r="E182" s="5" t="n"/>
     </row>
@@ -4105,7 +4105,7 @@
       </c>
       <c r="B183" s="5" t="inlineStr">
         <is>
-          <t>Purifying Shampoo 250 ml</t>
+          <t>Energizing Seasonal Superactive 100 ml</t>
         </is>
       </c>
       <c r="C183" s="5" t="inlineStr">
@@ -4114,7 +4114,7 @@
         </is>
       </c>
       <c r="D183" s="6" t="n">
-        <v>22.9</v>
+        <v>74</v>
       </c>
       <c r="E183" s="5" t="n"/>
     </row>
@@ -4124,7 +4124,7 @@
       </c>
       <c r="B184" s="5" t="inlineStr">
         <is>
-          <t>Purifying Shampoo 1000 ml</t>
+          <t>Energizing Seasonal Superactive 12x6 ml</t>
         </is>
       </c>
       <c r="C184" s="5" t="inlineStr">
@@ -4133,7 +4133,7 @@
         </is>
       </c>
       <c r="D184" s="6" t="n">
-        <v>68.7</v>
+        <v>74</v>
       </c>
       <c r="E184" s="5" t="n"/>
     </row>
@@ -4143,7 +4143,7 @@
       </c>
       <c r="B185" s="5" t="inlineStr">
         <is>
-          <t>Purifying Gel 150 ml</t>
+          <t>Energizing Superactive Anytime 100 ml</t>
         </is>
       </c>
       <c r="C185" s="5" t="inlineStr">
@@ -4152,7 +4152,7 @@
         </is>
       </c>
       <c r="D185" s="6" t="n">
-        <v>37.6</v>
+        <v>85</v>
       </c>
       <c r="E185" s="5" t="n"/>
     </row>
@@ -4162,7 +4162,7 @@
       </c>
       <c r="B186" s="5" t="inlineStr">
         <is>
-          <t>Well-Being Shampoo 100 ml</t>
+          <t>Energizing Gel 150 ml</t>
         </is>
       </c>
       <c r="C186" s="5" t="inlineStr">
@@ -4171,7 +4171,7 @@
         </is>
       </c>
       <c r="D186" s="6" t="n">
-        <v>13.3</v>
+        <v>37.6</v>
       </c>
       <c r="E186" s="5" t="n"/>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="B187" s="5" t="inlineStr">
         <is>
-          <t>Well-Being Shampoo 250 ml</t>
+          <t>Energizing Thickening Tonic 100 ml</t>
         </is>
       </c>
       <c r="C187" s="5" t="inlineStr">
@@ -4190,7 +4190,7 @@
         </is>
       </c>
       <c r="D187" s="6" t="n">
-        <v>22.9</v>
+        <v>44</v>
       </c>
       <c r="E187" s="5" t="n"/>
     </row>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="B188" s="5" t="inlineStr">
         <is>
-          <t>Well-Being Shampoo 1000 ml</t>
+          <t>Purifying Shampoo 100 ml</t>
         </is>
       </c>
       <c r="C188" s="5" t="inlineStr">
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="D188" s="6" t="n">
-        <v>68.7</v>
+        <v>13.3</v>
       </c>
       <c r="E188" s="5" t="n"/>
     </row>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="B189" s="5" t="inlineStr">
         <is>
-          <t>Well-Being Conditioner 60 ml</t>
+          <t>Purifying Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C189" s="5" t="inlineStr">
@@ -4228,7 +4228,7 @@
         </is>
       </c>
       <c r="D189" s="6" t="n">
-        <v>13.2</v>
+        <v>22.9</v>
       </c>
       <c r="E189" s="5" t="n"/>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="B190" s="5" t="inlineStr">
         <is>
-          <t>Well-Being Conditioner 150 ml</t>
+          <t>Purifying Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C190" s="5" t="inlineStr">
@@ -4247,7 +4247,7 @@
         </is>
       </c>
       <c r="D190" s="6" t="n">
-        <v>22.2</v>
+        <v>68.7</v>
       </c>
       <c r="E190" s="5" t="n"/>
     </row>
@@ -4257,7 +4257,7 @@
       </c>
       <c r="B191" s="5" t="inlineStr">
         <is>
-          <t>Well-Being Conditioner 1000 ml</t>
+          <t>Purifying Gel 150 ml</t>
         </is>
       </c>
       <c r="C191" s="5" t="inlineStr">
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="D191" s="6" t="n">
-        <v>87</v>
+        <v>37.6</v>
       </c>
       <c r="E191" s="5" t="n"/>
     </row>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="B192" s="5" t="inlineStr">
         <is>
-          <t>Detoxifying Scrub Shampoo 100 ml</t>
+          <t>Well-Being Shampoo 100 ml</t>
         </is>
       </c>
       <c r="C192" s="5" t="inlineStr">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="B193" s="5" t="inlineStr">
         <is>
-          <t>Detoxifying Scrub Shampoo 250 ml</t>
+          <t>Well-Being Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C193" s="5" t="inlineStr">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="B194" s="5" t="inlineStr">
         <is>
-          <t>Detoxifying Scrub Shampoo 1000 ml</t>
+          <t>Well-Being Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C194" s="5" t="inlineStr">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="B195" s="5" t="inlineStr">
         <is>
-          <t>Rebalancing Shampoo 100 ml</t>
+          <t>Well-Being Conditioner 60 ml</t>
         </is>
       </c>
       <c r="C195" s="5" t="inlineStr">
@@ -4342,7 +4342,7 @@
         </is>
       </c>
       <c r="D195" s="6" t="n">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
       <c r="E195" s="5" t="n"/>
     </row>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="B196" s="5" t="inlineStr">
         <is>
-          <t>Rebalancing Shampoo 250 ml</t>
+          <t>Well-Being Conditioner 150 ml</t>
         </is>
       </c>
       <c r="C196" s="5" t="inlineStr">
@@ -4361,7 +4361,7 @@
         </is>
       </c>
       <c r="D196" s="6" t="n">
-        <v>22.9</v>
+        <v>22.2</v>
       </c>
       <c r="E196" s="5" t="n"/>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="B197" s="5" t="inlineStr">
         <is>
-          <t>Rebalancing Shampoo 1000 ml</t>
+          <t>Well-Being Conditioner 1000 ml</t>
         </is>
       </c>
       <c r="C197" s="5" t="inlineStr">
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="D197" s="6" t="n">
-        <v>68.7</v>
+        <v>87</v>
       </c>
       <c r="E197" s="5" t="n"/>
     </row>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="B198" s="5" t="inlineStr">
         <is>
-          <t>Cleansing Treatment 250 ml</t>
+          <t>Detoxifying Scrub Shampoo 100 ml</t>
         </is>
       </c>
       <c r="C198" s="5" t="inlineStr">
@@ -4399,7 +4399,7 @@
         </is>
       </c>
       <c r="D198" s="6" t="n">
-        <v>28.1</v>
+        <v>13.3</v>
       </c>
       <c r="E198" s="5" t="n"/>
     </row>
@@ -4409,7 +4409,7 @@
       </c>
       <c r="B199" s="5" t="inlineStr">
         <is>
-          <t>Cleansing Treatment 1000 ml</t>
+          <t>Detoxifying Scrub Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C199" s="5" t="inlineStr">
@@ -4418,7 +4418,7 @@
         </is>
       </c>
       <c r="D199" s="6" t="n">
-        <v>84.7</v>
+        <v>22.9</v>
       </c>
       <c r="E199" s="5" t="n"/>
     </row>
@@ -4428,7 +4428,7 @@
       </c>
       <c r="B200" s="5" t="inlineStr">
         <is>
-          <t>Calming Shampoo 100 ml</t>
+          <t>Detoxifying Scrub Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C200" s="5" t="inlineStr">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D200" s="6" t="n">
-        <v>13.3</v>
+        <v>68.7</v>
       </c>
       <c r="E200" s="5" t="n"/>
     </row>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="B201" s="5" t="inlineStr">
         <is>
-          <t>Calming Shampoo 250 ml</t>
+          <t>Rebalancing Shampoo 100 ml</t>
         </is>
       </c>
       <c r="C201" s="5" t="inlineStr">
@@ -4456,7 +4456,7 @@
         </is>
       </c>
       <c r="D201" s="6" t="n">
-        <v>22.9</v>
+        <v>13.3</v>
       </c>
       <c r="E201" s="5" t="n"/>
     </row>
@@ -4466,7 +4466,7 @@
       </c>
       <c r="B202" s="5" t="inlineStr">
         <is>
-          <t>Calming Shampoo 1000 ml</t>
+          <t>Rebalancing Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C202" s="5" t="inlineStr">
@@ -4475,7 +4475,7 @@
         </is>
       </c>
       <c r="D202" s="6" t="n">
-        <v>68.7</v>
+        <v>22.9</v>
       </c>
       <c r="E202" s="5" t="n"/>
     </row>
@@ -4485,7 +4485,7 @@
       </c>
       <c r="B203" s="5" t="inlineStr">
         <is>
-          <t>Calming Superactive 100 ml</t>
+          <t>Rebalancing Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C203" s="5" t="inlineStr">
@@ -4494,7 +4494,7 @@
         </is>
       </c>
       <c r="D203" s="6" t="n">
-        <v>45.5</v>
+        <v>68.7</v>
       </c>
       <c r="E203" s="5" t="n"/>
     </row>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="B204" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Shampoo 100 ml</t>
+          <t>Cleansing Treatment 250 ml</t>
         </is>
       </c>
       <c r="C204" s="5" t="inlineStr">
@@ -4513,7 +4513,7 @@
         </is>
       </c>
       <c r="D204" s="6" t="n">
-        <v>13.3</v>
+        <v>28.1</v>
       </c>
       <c r="E204" s="5" t="n"/>
     </row>
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B205" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Shampoo 250 ml</t>
+          <t>Cleansing Treatment 1000 ml</t>
         </is>
       </c>
       <c r="C205" s="5" t="inlineStr">
@@ -4532,7 +4532,7 @@
         </is>
       </c>
       <c r="D205" s="6" t="n">
-        <v>22.9</v>
+        <v>84.7</v>
       </c>
       <c r="E205" s="5" t="n"/>
     </row>
@@ -4542,7 +4542,7 @@
       </c>
       <c r="B206" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Shampoo 1000 ml</t>
+          <t>Calming Shampoo 100 ml</t>
         </is>
       </c>
       <c r="C206" s="5" t="inlineStr">
@@ -4551,7 +4551,7 @@
         </is>
       </c>
       <c r="D206" s="6" t="n">
-        <v>68.7</v>
+        <v>13.3</v>
       </c>
       <c r="E206" s="5" t="n"/>
     </row>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="B207" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Vegetarian Miracle Conditioner 60 ml</t>
+          <t>Calming Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C207" s="5" t="inlineStr">
@@ -4570,7 +4570,7 @@
         </is>
       </c>
       <c r="D207" s="6" t="n">
-        <v>13.2</v>
+        <v>22.9</v>
       </c>
       <c r="E207" s="5" t="n"/>
     </row>
@@ -4580,7 +4580,7 @@
       </c>
       <c r="B208" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Vegetarian Miracle Conditioner 250 ml</t>
+          <t>Calming Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C208" s="5" t="inlineStr">
@@ -4589,7 +4589,7 @@
         </is>
       </c>
       <c r="D208" s="6" t="n">
-        <v>37.8</v>
+        <v>68.7</v>
       </c>
       <c r="E208" s="5" t="n"/>
     </row>
@@ -4599,7 +4599,7 @@
       </c>
       <c r="B209" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Vegetarian Miracle Conditioner 1000 ml</t>
+          <t>Calming Superactive 100 ml</t>
         </is>
       </c>
       <c r="C209" s="5" t="inlineStr">
@@ -4608,7 +4608,7 @@
         </is>
       </c>
       <c r="D209" s="6" t="n">
-        <v>113.4</v>
+        <v>45.5</v>
       </c>
       <c r="E209" s="5" t="n"/>
     </row>
@@ -4618,7 +4618,7 @@
       </c>
       <c r="B210" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Vegetarian Miracle Mask 60 ml</t>
+          <t>Nourishing Shampoo 100 ml</t>
         </is>
       </c>
       <c r="C210" s="5" t="inlineStr">
@@ -4627,7 +4627,7 @@
         </is>
       </c>
       <c r="D210" s="6" t="n">
-        <v>13.5</v>
+        <v>13.3</v>
       </c>
       <c r="E210" s="5" t="n"/>
     </row>
@@ -4637,7 +4637,7 @@
       </c>
       <c r="B211" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Vegetarian Miracle Mask 250 ml</t>
+          <t>Nourishing Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C211" s="5" t="inlineStr">
@@ -4646,7 +4646,7 @@
         </is>
       </c>
       <c r="D211" s="6" t="n">
-        <v>43</v>
+        <v>22.9</v>
       </c>
       <c r="E211" s="5" t="n"/>
     </row>
@@ -4656,7 +4656,7 @@
       </c>
       <c r="B212" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Vegetarian Miracle Mask 1000 ml</t>
+          <t>Nourishing Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C212" s="5" t="inlineStr">
@@ -4665,7 +4665,7 @@
         </is>
       </c>
       <c r="D212" s="6" t="n">
-        <v>129</v>
+        <v>68.7</v>
       </c>
       <c r="E212" s="5" t="n"/>
     </row>
@@ -4675,7 +4675,7 @@
       </c>
       <c r="B213" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Hair Building Pak 60 ml</t>
+          <t>Nourishing Vegetarian Miracle Conditioner 60 ml</t>
         </is>
       </c>
       <c r="C213" s="5" t="inlineStr">
@@ -4684,7 +4684,7 @@
         </is>
       </c>
       <c r="D213" s="6" t="n">
-        <v>13.7</v>
+        <v>13.2</v>
       </c>
       <c r="E213" s="5" t="n"/>
     </row>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="B214" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Hair Building Pak 250 ml</t>
+          <t>Nourishing Vegetarian Miracle Conditioner 250 ml</t>
         </is>
       </c>
       <c r="C214" s="5" t="inlineStr">
@@ -4703,7 +4703,7 @@
         </is>
       </c>
       <c r="D214" s="6" t="n">
-        <v>44.6</v>
+        <v>37.8</v>
       </c>
       <c r="E214" s="5" t="n"/>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="B215" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Keratin Sealer 100 ml</t>
+          <t>Nourishing Vegetarian Miracle Conditioner 1000 ml</t>
         </is>
       </c>
       <c r="C215" s="5" t="inlineStr">
@@ -4722,7 +4722,7 @@
         </is>
       </c>
       <c r="D215" s="6" t="n">
-        <v>38.2</v>
+        <v>113.4</v>
       </c>
       <c r="E215" s="5" t="n"/>
     </row>
@@ -4732,7 +4732,7 @@
       </c>
       <c r="B216" s="5" t="inlineStr">
         <is>
-          <t>Nourishing Hair Royal Jelly Superactive 6x8 ml</t>
+          <t>Nourishing Vegetarian Miracle Mask 60 ml</t>
         </is>
       </c>
       <c r="C216" s="5" t="inlineStr">
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="D216" s="6" t="n">
-        <v>79.59999999999999</v>
+        <v>13.5</v>
       </c>
       <c r="E216" s="5" t="n"/>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="B217" s="5" t="inlineStr">
         <is>
-          <t>Elevating Scalp Recovery Treatment 100 ml</t>
+          <t>Nourishing Vegetarian Miracle Mask 250 ml</t>
         </is>
       </c>
       <c r="C217" s="5" t="inlineStr">
@@ -4760,7 +4760,7 @@
         </is>
       </c>
       <c r="D217" s="6" t="n">
-        <v>48.8</v>
+        <v>43</v>
       </c>
       <c r="E217" s="5" t="n"/>
     </row>
@@ -4770,16 +4770,16 @@
       </c>
       <c r="B218" s="5" t="inlineStr">
         <is>
-          <t>OI/Shampoo 90 ml</t>
+          <t>Nourishing Vegetarian Miracle Mask 1000 ml</t>
         </is>
       </c>
       <c r="C218" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - OI</t>
+          <t>Prodotto - Naturaltech</t>
         </is>
       </c>
       <c r="D218" s="6" t="n">
-        <v>12.8</v>
+        <v>129</v>
       </c>
       <c r="E218" s="5" t="n"/>
     </row>
@@ -4789,16 +4789,16 @@
       </c>
       <c r="B219" s="5" t="inlineStr">
         <is>
-          <t>OI/Shampoo 280 ml</t>
+          <t>Nourishing Hair Building Pak 60 ml</t>
         </is>
       </c>
       <c r="C219" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - OI</t>
+          <t>Prodotto - Naturaltech</t>
         </is>
       </c>
       <c r="D219" s="6" t="n">
-        <v>22.6</v>
+        <v>13.7</v>
       </c>
       <c r="E219" s="5" t="n"/>
     </row>
@@ -4808,16 +4808,16 @@
       </c>
       <c r="B220" s="5" t="inlineStr">
         <is>
-          <t>OI/Shampoo 1000 ml</t>
+          <t>Nourishing Hair Building Pak 250 ml</t>
         </is>
       </c>
       <c r="C220" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - OI</t>
+          <t>Prodotto - Naturaltech</t>
         </is>
       </c>
       <c r="D220" s="6" t="n">
-        <v>67.8</v>
+        <v>44.6</v>
       </c>
       <c r="E220" s="5" t="n"/>
     </row>
@@ -4827,16 +4827,16 @@
       </c>
       <c r="B221" s="5" t="inlineStr">
         <is>
-          <t>OI/Conditioner 75 ml</t>
+          <t>Nourishing Keratin Sealer 100 ml</t>
         </is>
       </c>
       <c r="C221" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - OI</t>
+          <t>Prodotto - Naturaltech</t>
         </is>
       </c>
       <c r="D221" s="6" t="n">
-        <v>13.1</v>
+        <v>38.2</v>
       </c>
       <c r="E221" s="5" t="n"/>
     </row>
@@ -4846,16 +4846,16 @@
       </c>
       <c r="B222" s="5" t="inlineStr">
         <is>
-          <t>OI/Conditioner 250 ml</t>
+          <t>Nourishing Hair Royal Jelly Superactive 6x8 ml</t>
         </is>
       </c>
       <c r="C222" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - OI</t>
+          <t>Prodotto - Naturaltech</t>
         </is>
       </c>
       <c r="D222" s="6" t="n">
-        <v>30.2</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="E222" s="5" t="n"/>
     </row>
@@ -4865,16 +4865,16 @@
       </c>
       <c r="B223" s="5" t="inlineStr">
         <is>
-          <t>OI/Conditioner 1000 ml</t>
+          <t>Elevating Scalp Recovery Treatment 100 ml</t>
         </is>
       </c>
       <c r="C223" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - OI</t>
+          <t>Prodotto - Naturaltech</t>
         </is>
       </c>
       <c r="D223" s="6" t="n">
-        <v>90.59999999999999</v>
+        <v>48.8</v>
       </c>
       <c r="E223" s="5" t="n"/>
     </row>
@@ -4884,7 +4884,7 @@
       </c>
       <c r="B224" s="5" t="inlineStr">
         <is>
-          <t>OI/Hair Butter 75 ml</t>
+          <t>OI/Shampoo 90 ml</t>
         </is>
       </c>
       <c r="C224" s="5" t="inlineStr">
@@ -4893,7 +4893,7 @@
         </is>
       </c>
       <c r="D224" s="6" t="n">
-        <v>14.2</v>
+        <v>12.8</v>
       </c>
       <c r="E224" s="5" t="n"/>
     </row>
@@ -4903,7 +4903,7 @@
       </c>
       <c r="B225" s="5" t="inlineStr">
         <is>
-          <t>OI/Hair Butter 250 ml</t>
+          <t>OI/Shampoo 280 ml</t>
         </is>
       </c>
       <c r="C225" s="5" t="inlineStr">
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="D225" s="6" t="n">
-        <v>34</v>
+        <v>22.6</v>
       </c>
       <c r="E225" s="5" t="n"/>
     </row>
@@ -4922,7 +4922,7 @@
       </c>
       <c r="B226" s="5" t="inlineStr">
         <is>
-          <t>OI/Hair Butter 1000 ml</t>
+          <t>OI/Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C226" s="5" t="inlineStr">
@@ -4931,7 +4931,7 @@
         </is>
       </c>
       <c r="D226" s="6" t="n">
-        <v>102</v>
+        <v>67.8</v>
       </c>
       <c r="E226" s="5" t="n"/>
     </row>
@@ -4941,7 +4941,7 @@
       </c>
       <c r="B227" s="5" t="inlineStr">
         <is>
-          <t>OI/Oil 50 ml</t>
+          <t>OI/Conditioner 75 ml</t>
         </is>
       </c>
       <c r="C227" s="5" t="inlineStr">
@@ -4950,7 +4950,7 @@
         </is>
       </c>
       <c r="D227" s="6" t="n">
-        <v>25.9</v>
+        <v>13.1</v>
       </c>
       <c r="E227" s="5" t="n"/>
     </row>
@@ -4960,7 +4960,7 @@
       </c>
       <c r="B228" s="5" t="inlineStr">
         <is>
-          <t>OI/Oil 135 ml</t>
+          <t>OI/Conditioner 250 ml</t>
         </is>
       </c>
       <c r="C228" s="5" t="inlineStr">
@@ -4969,7 +4969,7 @@
         </is>
       </c>
       <c r="D228" s="6" t="n">
-        <v>46.2</v>
+        <v>30.2</v>
       </c>
       <c r="E228" s="5" t="n"/>
     </row>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="B229" s="5" t="inlineStr">
         <is>
-          <t>OI/Liquid Luster 100 ml</t>
+          <t>OI/Conditioner 1000 ml</t>
         </is>
       </c>
       <c r="C229" s="5" t="inlineStr">
@@ -4988,7 +4988,7 @@
         </is>
       </c>
       <c r="D229" s="6" t="n">
-        <v>25</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="E229" s="5" t="n"/>
     </row>
@@ -4998,7 +4998,7 @@
       </c>
       <c r="B230" s="5" t="inlineStr">
         <is>
-          <t>OI/Liquid Luster 300 ml</t>
+          <t>OI/Hair Butter 75 ml</t>
         </is>
       </c>
       <c r="C230" s="5" t="inlineStr">
@@ -5007,7 +5007,7 @@
         </is>
       </c>
       <c r="D230" s="6" t="n">
-        <v>42</v>
+        <v>14.2</v>
       </c>
       <c r="E230" s="5" t="n"/>
     </row>
@@ -5017,7 +5017,7 @@
       </c>
       <c r="B231" s="5" t="inlineStr">
         <is>
-          <t>OI/All in One Milk 50 ml</t>
+          <t>OI/Hair Butter 250 ml</t>
         </is>
       </c>
       <c r="C231" s="5" t="inlineStr">
@@ -5026,7 +5026,7 @@
         </is>
       </c>
       <c r="D231" s="6" t="n">
-        <v>20.2</v>
+        <v>34</v>
       </c>
       <c r="E231" s="5" t="n"/>
     </row>
@@ -5036,7 +5036,7 @@
       </c>
       <c r="B232" s="5" t="inlineStr">
         <is>
-          <t>OI/All in One Milk 135 ml</t>
+          <t>OI/Hair Butter 1000 ml</t>
         </is>
       </c>
       <c r="C232" s="5" t="inlineStr">
@@ -5045,7 +5045,7 @@
         </is>
       </c>
       <c r="D232" s="6" t="n">
-        <v>30.4</v>
+        <v>102</v>
       </c>
       <c r="E232" s="5" t="n"/>
     </row>
@@ -5055,7 +5055,7 @@
       </c>
       <c r="B233" s="5" t="inlineStr">
         <is>
-          <t>OI/Body Wash 90 ml</t>
+          <t>OI/Oil 50 ml</t>
         </is>
       </c>
       <c r="C233" s="5" t="inlineStr">
@@ -5064,7 +5064,7 @@
         </is>
       </c>
       <c r="D233" s="6" t="n">
-        <v>12.4</v>
+        <v>25.9</v>
       </c>
       <c r="E233" s="5" t="n"/>
     </row>
@@ -5074,7 +5074,7 @@
       </c>
       <c r="B234" s="5" t="inlineStr">
         <is>
-          <t>OI/Body Wash 280 ml</t>
+          <t>OI/Oil 135 ml</t>
         </is>
       </c>
       <c r="C234" s="5" t="inlineStr">
@@ -5083,7 +5083,7 @@
         </is>
       </c>
       <c r="D234" s="6" t="n">
-        <v>19.8</v>
+        <v>46.2</v>
       </c>
       <c r="E234" s="5" t="n"/>
     </row>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="B235" s="5" t="inlineStr">
         <is>
-          <t>OI/Hand Balm 75 ml</t>
+          <t>OI/Liquid Luster 100 ml</t>
         </is>
       </c>
       <c r="C235" s="5" t="inlineStr">
@@ -5102,7 +5102,7 @@
         </is>
       </c>
       <c r="D235" s="6" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E235" s="5" t="n"/>
     </row>
@@ -5112,16 +5112,16 @@
       </c>
       <c r="B236" s="5" t="inlineStr">
         <is>
-          <t>Softening Shaving Gel 200 ml</t>
+          <t>OI/Liquid Luster 300 ml</t>
         </is>
       </c>
       <c r="C236" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Pasta &amp; Love</t>
+          <t>Prodotto - OI</t>
         </is>
       </c>
       <c r="D236" s="6" t="n">
-        <v>31.3</v>
+        <v>42</v>
       </c>
       <c r="E236" s="5" t="n"/>
     </row>
@@ -5131,16 +5131,16 @@
       </c>
       <c r="B237" s="5" t="inlineStr">
         <is>
-          <t>After Shave &amp; Moisturizing Cream 100 ml</t>
+          <t>OI/All in One Milk 50 ml</t>
         </is>
       </c>
       <c r="C237" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Pasta &amp; Love</t>
+          <t>Prodotto - OI</t>
         </is>
       </c>
       <c r="D237" s="6" t="n">
-        <v>33</v>
+        <v>20.2</v>
       </c>
       <c r="E237" s="5" t="n"/>
     </row>
@@ -5150,16 +5150,16 @@
       </c>
       <c r="B238" s="5" t="inlineStr">
         <is>
-          <t>Pre-Shaving &amp; Beard Oil 50 ml</t>
+          <t>OI/All in One Milk 135 ml</t>
         </is>
       </c>
       <c r="C238" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Pasta &amp; Love</t>
+          <t>Prodotto - OI</t>
         </is>
       </c>
       <c r="D238" s="6" t="n">
-        <v>30.2</v>
+        <v>30.4</v>
       </c>
       <c r="E238" s="5" t="n"/>
     </row>
@@ -5169,16 +5169,16 @@
       </c>
       <c r="B239" s="5" t="inlineStr">
         <is>
-          <t>Medium Hold Styling Paste 125 ml</t>
+          <t>OI/Body Wash 90 ml</t>
         </is>
       </c>
       <c r="C239" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Pasta &amp; Love</t>
+          <t>Prodotto - OI</t>
         </is>
       </c>
       <c r="D239" s="6" t="n">
-        <v>28.9</v>
+        <v>12.4</v>
       </c>
       <c r="E239" s="5" t="n"/>
     </row>
@@ -5188,16 +5188,16 @@
       </c>
       <c r="B240" s="5" t="inlineStr">
         <is>
-          <t>Non-Foaming Transparent Shaving Gel 150 ml</t>
+          <t>OI/Body Wash 280 ml</t>
         </is>
       </c>
       <c r="C240" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Pasta &amp; Love</t>
+          <t>Prodotto - OI</t>
         </is>
       </c>
       <c r="D240" s="6" t="n">
-        <v>25</v>
+        <v>19.8</v>
       </c>
       <c r="E240" s="5" t="n"/>
     </row>
@@ -5207,16 +5207,16 @@
       </c>
       <c r="B241" s="5" t="inlineStr">
         <is>
-          <t>Strong-Hold Mat Clay 50 ml</t>
+          <t>OI/Hand Balm 75 ml</t>
         </is>
       </c>
       <c r="C241" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Pasta &amp; Love</t>
+          <t>Prodotto - OI</t>
         </is>
       </c>
       <c r="D241" s="6" t="n">
-        <v>18.2</v>
+        <v>18</v>
       </c>
       <c r="E241" s="5" t="n"/>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="B242" s="5" t="inlineStr">
         <is>
-          <t>Hair Beard &amp; Body Wash 300 ml</t>
+          <t>Softening Shaving Gel 200 ml</t>
         </is>
       </c>
       <c r="C242" s="5" t="inlineStr">
@@ -5235,7 +5235,7 @@
         </is>
       </c>
       <c r="D242" s="6" t="n">
-        <v>22.6</v>
+        <v>31.3</v>
       </c>
       <c r="E242" s="5" t="n"/>
     </row>
@@ -5245,7 +5245,7 @@
       </c>
       <c r="B243" s="5" t="inlineStr">
         <is>
-          <t>Fiber Cream 50 ml</t>
+          <t>After Shave &amp; Moisturizing Cream 100 ml</t>
         </is>
       </c>
       <c r="C243" s="5" t="inlineStr">
@@ -5254,7 +5254,7 @@
         </is>
       </c>
       <c r="D243" s="6" t="n">
-        <v>22.9</v>
+        <v>33</v>
       </c>
       <c r="E243" s="5" t="n"/>
     </row>
@@ -5264,16 +5264,16 @@
       </c>
       <c r="B244" s="5" t="inlineStr">
         <is>
-          <t>Silkening Shampoo 90 ml</t>
+          <t>Pre-Shaving &amp; Beard Oil 50 ml</t>
         </is>
       </c>
       <c r="C244" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Heart of Glass</t>
+          <t>Prodotto - Pasta &amp; Love</t>
         </is>
       </c>
       <c r="D244" s="6" t="n">
-        <v>11.7</v>
+        <v>30.2</v>
       </c>
       <c r="E244" s="5" t="n"/>
     </row>
@@ -5283,16 +5283,16 @@
       </c>
       <c r="B245" s="5" t="inlineStr">
         <is>
-          <t>Silkening Shampoo 250 ml</t>
+          <t>Medium Hold Styling Paste 125 ml</t>
         </is>
       </c>
       <c r="C245" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Heart of Glass</t>
+          <t>Prodotto - Pasta &amp; Love</t>
         </is>
       </c>
       <c r="D245" s="6" t="n">
-        <v>20.8</v>
+        <v>28.9</v>
       </c>
       <c r="E245" s="5" t="n"/>
     </row>
@@ -5302,16 +5302,16 @@
       </c>
       <c r="B246" s="5" t="inlineStr">
         <is>
-          <t>Silkening Shampoo 1000 ml</t>
+          <t>Non-Foaming Transparent Shaving Gel 150 ml</t>
         </is>
       </c>
       <c r="C246" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Heart of Glass</t>
+          <t>Prodotto - Pasta &amp; Love</t>
         </is>
       </c>
       <c r="D246" s="6" t="n">
-        <v>62.4</v>
+        <v>25</v>
       </c>
       <c r="E246" s="5" t="n"/>
     </row>
@@ -5321,16 +5321,16 @@
       </c>
       <c r="B247" s="5" t="inlineStr">
         <is>
-          <t>Rich Conditioner 90 ml</t>
+          <t>Strong-Hold Mat Clay 50 ml</t>
         </is>
       </c>
       <c r="C247" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Heart of Glass</t>
+          <t>Prodotto - Pasta &amp; Love</t>
         </is>
       </c>
       <c r="D247" s="6" t="n">
-        <v>12.9</v>
+        <v>18.2</v>
       </c>
       <c r="E247" s="5" t="n"/>
     </row>
@@ -5340,16 +5340,16 @@
       </c>
       <c r="B248" s="5" t="inlineStr">
         <is>
-          <t>Rich Conditioner 250 ml</t>
+          <t>Hair Beard &amp; Body Wash 300 ml</t>
         </is>
       </c>
       <c r="C248" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Heart of Glass</t>
+          <t>Prodotto - Pasta &amp; Love</t>
         </is>
       </c>
       <c r="D248" s="6" t="n">
-        <v>30.2</v>
+        <v>22.6</v>
       </c>
       <c r="E248" s="5" t="n"/>
     </row>
@@ -5359,16 +5359,16 @@
       </c>
       <c r="B249" s="5" t="inlineStr">
         <is>
-          <t>Rich Conditioner 1000 ml</t>
+          <t>Fiber Cream 50 ml</t>
         </is>
       </c>
       <c r="C249" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Heart of Glass</t>
+          <t>Prodotto - Pasta &amp; Love</t>
         </is>
       </c>
       <c r="D249" s="6" t="n">
-        <v>90.59999999999999</v>
+        <v>22.9</v>
       </c>
       <c r="E249" s="5" t="n"/>
     </row>
@@ -5378,7 +5378,7 @@
       </c>
       <c r="B250" s="5" t="inlineStr">
         <is>
-          <t>Intense Treatment 150 ml</t>
+          <t>Silkening Shampoo 90 ml</t>
         </is>
       </c>
       <c r="C250" s="5" t="inlineStr">
@@ -5387,7 +5387,7 @@
         </is>
       </c>
       <c r="D250" s="6" t="n">
-        <v>28.6</v>
+        <v>11.7</v>
       </c>
       <c r="E250" s="5" t="n"/>
     </row>
@@ -5397,7 +5397,7 @@
       </c>
       <c r="B251" s="5" t="inlineStr">
         <is>
-          <t>Sheer Glaze 150 ml</t>
+          <t>Silkening Shampoo 250 ml</t>
         </is>
       </c>
       <c r="C251" s="5" t="inlineStr">
@@ -5406,7 +5406,7 @@
         </is>
       </c>
       <c r="D251" s="6" t="n">
-        <v>30.4</v>
+        <v>20.8</v>
       </c>
       <c r="E251" s="5" t="n"/>
     </row>
@@ -5416,7 +5416,7 @@
       </c>
       <c r="B252" s="5" t="inlineStr">
         <is>
-          <t>Instant Bonding Glow 300 ml</t>
+          <t>Silkening Shampoo 1000 ml</t>
         </is>
       </c>
       <c r="C252" s="5" t="inlineStr">
@@ -5425,7 +5425,7 @@
         </is>
       </c>
       <c r="D252" s="6" t="n">
-        <v>42</v>
+        <v>62.4</v>
       </c>
       <c r="E252" s="5" t="n"/>
     </row>
@@ -5435,16 +5435,16 @@
       </c>
       <c r="B253" s="5" t="inlineStr">
         <is>
-          <t>Spray al Sale Marino 100 ml</t>
+          <t>Rich Conditioner 90 ml</t>
         </is>
       </c>
       <c r="C253" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - More Inside</t>
+          <t>Prodotto - Heart of Glass</t>
         </is>
       </c>
       <c r="D253" s="6" t="n">
-        <v>16.2</v>
+        <v>12.9</v>
       </c>
       <c r="E253" s="5" t="n"/>
     </row>
@@ -5454,16 +5454,16 @@
       </c>
       <c r="B254" s="5" t="inlineStr">
         <is>
-          <t>Spray al Sale Marino 250 ml</t>
+          <t>Rich Conditioner 250 ml</t>
         </is>
       </c>
       <c r="C254" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - More Inside</t>
+          <t>Prodotto - Heart of Glass</t>
         </is>
       </c>
       <c r="D254" s="6" t="n">
-        <v>32</v>
+        <v>30.2</v>
       </c>
       <c r="E254" s="5" t="n"/>
     </row>
@@ -5473,16 +5473,16 @@
       </c>
       <c r="B255" s="5" t="inlineStr">
         <is>
-          <t>Siero Crea Ricci 100 ml</t>
+          <t>Rich Conditioner 1000 ml</t>
         </is>
       </c>
       <c r="C255" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - More Inside</t>
+          <t>Prodotto - Heart of Glass</t>
         </is>
       </c>
       <c r="D255" s="6" t="n">
-        <v>16.2</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="E255" s="5" t="n"/>
     </row>
@@ -5492,16 +5492,16 @@
       </c>
       <c r="B256" s="5" t="inlineStr">
         <is>
-          <t>Siero Crea Ricci 250 ml</t>
+          <t>Intense Treatment 150 ml</t>
         </is>
       </c>
       <c r="C256" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - More Inside</t>
+          <t>Prodotto - Heart of Glass</t>
         </is>
       </c>
       <c r="D256" s="6" t="n">
-        <v>32</v>
+        <v>28.6</v>
       </c>
       <c r="E256" s="5" t="n"/>
     </row>
@@ -5511,16 +5511,16 @@
       </c>
       <c r="B257" s="5" t="inlineStr">
         <is>
-          <t>Oil Non Oil 250 ml</t>
+          <t>Sheer Glaze 150 ml</t>
         </is>
       </c>
       <c r="C257" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - More Inside</t>
+          <t>Prodotto - Heart of Glass</t>
         </is>
       </c>
       <c r="D257" s="6" t="n">
-        <v>28.7</v>
+        <v>30.4</v>
       </c>
       <c r="E257" s="5" t="n"/>
     </row>
@@ -5530,16 +5530,16 @@
       </c>
       <c r="B258" s="5" t="inlineStr">
         <is>
-          <t>Gel Medio Modellante 250 ml</t>
+          <t>Instant Bonding Glow 300 ml</t>
         </is>
       </c>
       <c r="C258" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - More Inside</t>
+          <t>Prodotto - Heart of Glass</t>
         </is>
       </c>
       <c r="D258" s="6" t="n">
-        <v>28.7</v>
+        <v>42</v>
       </c>
       <c r="E258" s="5" t="n"/>
     </row>
@@ -5549,7 +5549,7 @@
       </c>
       <c r="B259" s="5" t="inlineStr">
         <is>
-          <t>Gel Oil per i Ricci 250 ml</t>
+          <t>Spray al Sale Marino 100 ml</t>
         </is>
       </c>
       <c r="C259" s="5" t="inlineStr">
@@ -5558,7 +5558,7 @@
         </is>
       </c>
       <c r="D259" s="6" t="n">
-        <v>32</v>
+        <v>16.2</v>
       </c>
       <c r="E259" s="5" t="n"/>
     </row>
@@ -5568,7 +5568,7 @@
       </c>
       <c r="B260" s="5" t="inlineStr">
         <is>
-          <t>Blow Dry Primer 100 ml</t>
+          <t>Spray al Sale Marino 250 ml</t>
         </is>
       </c>
       <c r="C260" s="5" t="inlineStr">
@@ -5577,7 +5577,7 @@
         </is>
       </c>
       <c r="D260" s="6" t="n">
-        <v>15.1</v>
+        <v>32</v>
       </c>
       <c r="E260" s="5" t="n"/>
     </row>
@@ -5587,7 +5587,7 @@
       </c>
       <c r="B261" s="5" t="inlineStr">
         <is>
-          <t>Blow Dry Primer 250 ml</t>
+          <t>Siero Crea Ricci 100 ml</t>
         </is>
       </c>
       <c r="C261" s="5" t="inlineStr">
@@ -5596,7 +5596,7 @@
         </is>
       </c>
       <c r="D261" s="6" t="n">
-        <v>34.4</v>
+        <v>16.2</v>
       </c>
       <c r="E261" s="5" t="n"/>
     </row>
@@ -5606,7 +5606,7 @@
       </c>
       <c r="B262" s="5" t="inlineStr">
         <is>
-          <t>Siero Texturizzante 150 ml</t>
+          <t>Siero Crea Ricci 250 ml</t>
         </is>
       </c>
       <c r="C262" s="5" t="inlineStr">
@@ -5615,7 +5615,7 @@
         </is>
       </c>
       <c r="D262" s="6" t="n">
-        <v>27.2</v>
+        <v>32</v>
       </c>
       <c r="E262" s="5" t="n"/>
     </row>
@@ -5625,7 +5625,7 @@
       </c>
       <c r="B263" s="5" t="inlineStr">
         <is>
-          <t>Polvere Texturizzante 8 gr</t>
+          <t>Oil Non Oil 250 ml</t>
         </is>
       </c>
       <c r="C263" s="5" t="inlineStr">
@@ -5634,7 +5634,7 @@
         </is>
       </c>
       <c r="D263" s="6" t="n">
-        <v>28.8</v>
+        <v>28.7</v>
       </c>
       <c r="E263" s="5" t="n"/>
     </row>
@@ -5644,7 +5644,7 @@
       </c>
       <c r="B264" s="5" t="inlineStr">
         <is>
-          <t>Siero Invisibile 50 ml</t>
+          <t>Gel Medio Modellante 250 ml</t>
         </is>
       </c>
       <c r="C264" s="5" t="inlineStr">
@@ -5653,7 +5653,7 @@
         </is>
       </c>
       <c r="D264" s="6" t="n">
-        <v>20.6</v>
+        <v>28.7</v>
       </c>
       <c r="E264" s="5" t="n"/>
     </row>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B265" s="5" t="inlineStr">
         <is>
-          <t>Fluido Stirante Idratante 125 ml</t>
+          <t>Gel Oil per i Ricci 250 ml</t>
         </is>
       </c>
       <c r="C265" s="5" t="inlineStr">
@@ -5672,7 +5672,7 @@
         </is>
       </c>
       <c r="D265" s="6" t="n">
-        <v>21.9</v>
+        <v>32</v>
       </c>
       <c r="E265" s="5" t="n"/>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="B266" s="5" t="inlineStr">
         <is>
-          <t>Crema Gel Forte 125 ml</t>
+          <t>Blow Dry Primer 100 ml</t>
         </is>
       </c>
       <c r="C266" s="5" t="inlineStr">
@@ -5691,7 +5691,7 @@
         </is>
       </c>
       <c r="D266" s="6" t="n">
-        <v>19.6</v>
+        <v>15.1</v>
       </c>
       <c r="E266" s="5" t="n"/>
     </row>
@@ -5701,7 +5701,7 @@
       </c>
       <c r="B267" s="5" t="inlineStr">
         <is>
-          <t>Pasta Duttile Media 125 ml</t>
+          <t>Blow Dry Primer 250 ml</t>
         </is>
       </c>
       <c r="C267" s="5" t="inlineStr">
@@ -5710,7 +5710,7 @@
         </is>
       </c>
       <c r="D267" s="6" t="n">
-        <v>28.8</v>
+        <v>34.4</v>
       </c>
       <c r="E267" s="5" t="n"/>
     </row>
@@ -5720,7 +5720,7 @@
       </c>
       <c r="B268" s="5" t="inlineStr">
         <is>
-          <t>Lacca Media 400 ml</t>
+          <t>Siero Texturizzante 150 ml</t>
         </is>
       </c>
       <c r="C268" s="5" t="inlineStr">
@@ -5729,7 +5729,7 @@
         </is>
       </c>
       <c r="D268" s="6" t="n">
-        <v>29</v>
+        <v>27.2</v>
       </c>
       <c r="E268" s="5" t="n"/>
     </row>
@@ -5739,7 +5739,7 @@
       </c>
       <c r="B269" s="5" t="inlineStr">
         <is>
-          <t>Lacca Forte 100 ml</t>
+          <t>Polvere Texturizzante 8 gr</t>
         </is>
       </c>
       <c r="C269" s="5" t="inlineStr">
@@ -5748,7 +5748,7 @@
         </is>
       </c>
       <c r="D269" s="6" t="n">
-        <v>13.2</v>
+        <v>28.8</v>
       </c>
       <c r="E269" s="5" t="n"/>
     </row>
@@ -5758,7 +5758,7 @@
       </c>
       <c r="B270" s="5" t="inlineStr">
         <is>
-          <t>Lacca Forte 400 ml</t>
+          <t>Siero Invisibile 50 ml</t>
         </is>
       </c>
       <c r="C270" s="5" t="inlineStr">
@@ -5767,7 +5767,7 @@
         </is>
       </c>
       <c r="D270" s="6" t="n">
-        <v>29</v>
+        <v>20.6</v>
       </c>
       <c r="E270" s="5" t="n"/>
     </row>
@@ -5777,7 +5777,7 @@
       </c>
       <c r="B271" s="5" t="inlineStr">
         <is>
-          <t>Lacca Extra Forte 400 ml</t>
+          <t>Fluido Stirante Idratante 125 ml</t>
         </is>
       </c>
       <c r="C271" s="5" t="inlineStr">
@@ -5786,7 +5786,7 @@
         </is>
       </c>
       <c r="D271" s="6" t="n">
-        <v>32.3</v>
+        <v>21.9</v>
       </c>
       <c r="E271" s="5" t="n"/>
     </row>
@@ -5796,7 +5796,7 @@
       </c>
       <c r="B272" s="5" t="inlineStr">
         <is>
-          <t>Eco Lacca Invisibile 250 ml</t>
+          <t>Crema Gel Forte 125 ml</t>
         </is>
       </c>
       <c r="C272" s="5" t="inlineStr">
@@ -5805,7 +5805,7 @@
         </is>
       </c>
       <c r="D272" s="6" t="n">
-        <v>29</v>
+        <v>19.6</v>
       </c>
       <c r="E272" s="5" t="n"/>
     </row>
@@ -5815,7 +5815,7 @@
       </c>
       <c r="B273" s="5" t="inlineStr">
         <is>
-          <t>Spray Lucidante 200 ml</t>
+          <t>Pasta Duttile Media 125 ml</t>
         </is>
       </c>
       <c r="C273" s="5" t="inlineStr">
@@ -5824,7 +5824,7 @@
         </is>
       </c>
       <c r="D273" s="6" t="n">
-        <v>31.8</v>
+        <v>28.8</v>
       </c>
       <c r="E273" s="5" t="n"/>
     </row>
@@ -5834,7 +5834,7 @@
       </c>
       <c r="B274" s="5" t="inlineStr">
         <is>
-          <t>Mousse Volume 250 ml</t>
+          <t>Lacca Media 400 ml</t>
         </is>
       </c>
       <c r="C274" s="5" t="inlineStr">
@@ -5843,7 +5843,7 @@
         </is>
       </c>
       <c r="D274" s="6" t="n">
-        <v>25.5</v>
+        <v>29</v>
       </c>
       <c r="E274" s="5" t="n"/>
     </row>
@@ -5853,7 +5853,7 @@
       </c>
       <c r="B275" s="5" t="inlineStr">
         <is>
-          <t>Mousse Idratante Ricci 250 ml</t>
+          <t>Lacca Forte 100 ml</t>
         </is>
       </c>
       <c r="C275" s="5" t="inlineStr">
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D275" s="6" t="n">
-        <v>25.5</v>
+        <v>13.2</v>
       </c>
       <c r="E275" s="5" t="n"/>
     </row>
@@ -5872,7 +5872,7 @@
       </c>
       <c r="B276" s="5" t="inlineStr">
         <is>
-          <t>Spray Texturizzante Secco 250 ml</t>
+          <t>Lacca Forte 400 ml</t>
         </is>
       </c>
       <c r="C276" s="5" t="inlineStr">
@@ -5881,7 +5881,7 @@
         </is>
       </c>
       <c r="D276" s="6" t="n">
-        <v>30.5</v>
+        <v>29</v>
       </c>
       <c r="E276" s="5" t="n"/>
     </row>
@@ -5891,7 +5891,7 @@
       </c>
       <c r="B277" s="5" t="inlineStr">
         <is>
-          <t>Shampoo Secco Invisibile 250 ml</t>
+          <t>Lacca Extra Forte 400 ml</t>
         </is>
       </c>
       <c r="C277" s="5" t="inlineStr">
@@ -5900,7 +5900,7 @@
         </is>
       </c>
       <c r="D277" s="6" t="n">
-        <v>30.6</v>
+        <v>32.3</v>
       </c>
       <c r="E277" s="5" t="n"/>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="B278" s="5" t="inlineStr">
         <is>
-          <t>Cera Illuminante 75 ml</t>
+          <t>Eco Lacca Invisibile 250 ml</t>
         </is>
       </c>
       <c r="C278" s="5" t="inlineStr">
@@ -5919,7 +5919,7 @@
         </is>
       </c>
       <c r="D278" s="6" t="n">
-        <v>24.2</v>
+        <v>29</v>
       </c>
       <c r="E278" s="5" t="n"/>
     </row>
@@ -5929,7 +5929,7 @@
       </c>
       <c r="B279" s="5" t="inlineStr">
         <is>
-          <t>Pomade per Plasmare 75 ml</t>
+          <t>Spray Lucidante 200 ml</t>
         </is>
       </c>
       <c r="C279" s="5" t="inlineStr">
@@ -5938,7 +5938,7 @@
         </is>
       </c>
       <c r="D279" s="6" t="n">
-        <v>24.2</v>
+        <v>31.8</v>
       </c>
       <c r="E279" s="5" t="n"/>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="B280" s="5" t="inlineStr">
         <is>
-          <t>Gomma Texturizzante Media 75 ml</t>
+          <t>Mousse Volume 250 ml</t>
         </is>
       </c>
       <c r="C280" s="5" t="inlineStr">
@@ -5957,7 +5957,7 @@
         </is>
       </c>
       <c r="D280" s="6" t="n">
-        <v>24.2</v>
+        <v>25.5</v>
       </c>
       <c r="E280" s="5" t="n"/>
     </row>
@@ -5967,7 +5967,7 @@
       </c>
       <c r="B281" s="5" t="inlineStr">
         <is>
-          <t>Argilla Modellante Forte 75 ml</t>
+          <t>Mousse Idratante Ricci 250 ml</t>
         </is>
       </c>
       <c r="C281" s="5" t="inlineStr">
@@ -5976,7 +5976,7 @@
         </is>
       </c>
       <c r="D281" s="6" t="n">
-        <v>24.2</v>
+        <v>25.5</v>
       </c>
       <c r="E281" s="5" t="n"/>
     </row>
@@ -5986,7 +5986,7 @@
       </c>
       <c r="B282" s="5" t="inlineStr">
         <is>
-          <t>Cera Forte Asciutta 75 ml</t>
+          <t>Spray Texturizzante Secco 250 ml</t>
         </is>
       </c>
       <c r="C282" s="5" t="inlineStr">
@@ -5995,7 +5995,7 @@
         </is>
       </c>
       <c r="D282" s="6" t="n">
-        <v>24.2</v>
+        <v>30.5</v>
       </c>
       <c r="E282" s="5" t="n"/>
     </row>
@@ -6005,7 +6005,7 @@
       </c>
       <c r="B283" s="5" t="inlineStr">
         <is>
-          <t>Dry Wax 200 ml</t>
+          <t>Shampoo Secco Invisibile 250 ml</t>
         </is>
       </c>
       <c r="C283" s="5" t="inlineStr">
@@ -6014,7 +6014,7 @@
         </is>
       </c>
       <c r="D283" s="6" t="n">
-        <v>25.5</v>
+        <v>30.6</v>
       </c>
       <c r="E283" s="5" t="n"/>
     </row>
@@ -6024,16 +6024,16 @@
       </c>
       <c r="B284" s="5" t="inlineStr">
         <is>
-          <t>SU/Hair &amp; Body Wash 75 ml</t>
+          <t>Cera Illuminante 75 ml</t>
         </is>
       </c>
       <c r="C284" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - SU</t>
+          <t>Prodotto - More Inside</t>
         </is>
       </c>
       <c r="D284" s="6" t="n">
-        <v>9.4</v>
+        <v>24.2</v>
       </c>
       <c r="E284" s="5" t="n"/>
     </row>
@@ -6043,16 +6043,16 @@
       </c>
       <c r="B285" s="5" t="inlineStr">
         <is>
-          <t>SU/Hair &amp; Body Wash 500 ml</t>
+          <t>Pomade per Plasmare 75 ml</t>
         </is>
       </c>
       <c r="C285" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - SU</t>
+          <t>Prodotto - More Inside</t>
         </is>
       </c>
       <c r="D285" s="6" t="n">
-        <v>36</v>
+        <v>24.2</v>
       </c>
       <c r="E285" s="5" t="n"/>
     </row>
@@ -6062,16 +6062,16 @@
       </c>
       <c r="B286" s="5" t="inlineStr">
         <is>
-          <t>SU/Hair Mask 150 ml</t>
+          <t>Gomma Texturizzante Media 75 ml</t>
         </is>
       </c>
       <c r="C286" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - SU</t>
+          <t>Prodotto - More Inside</t>
         </is>
       </c>
       <c r="D286" s="6" t="n">
-        <v>22.4</v>
+        <v>24.2</v>
       </c>
       <c r="E286" s="5" t="n"/>
     </row>
@@ -6081,16 +6081,16 @@
       </c>
       <c r="B287" s="5" t="inlineStr">
         <is>
-          <t>SU/Hair Milk 50 ml</t>
+          <t>Argilla Modellante Forte 75 ml</t>
         </is>
       </c>
       <c r="C287" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - SU</t>
+          <t>Prodotto - More Inside</t>
         </is>
       </c>
       <c r="D287" s="6" t="n">
-        <v>14</v>
+        <v>24.2</v>
       </c>
       <c r="E287" s="5" t="n"/>
     </row>
@@ -6100,16 +6100,16 @@
       </c>
       <c r="B288" s="5" t="inlineStr">
         <is>
-          <t>SU/Hair Milk 135 ml</t>
+          <t>Cera Forte Asciutta 75 ml</t>
         </is>
       </c>
       <c r="C288" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - SU</t>
+          <t>Prodotto - More Inside</t>
         </is>
       </c>
       <c r="D288" s="6" t="n">
-        <v>22.4</v>
+        <v>24.2</v>
       </c>
       <c r="E288" s="5" t="n"/>
     </row>
@@ -6119,16 +6119,16 @@
       </c>
       <c r="B289" s="5" t="inlineStr">
         <is>
-          <t>SU/Tan Maximizer 150 ml</t>
+          <t>Dry Wax 200 ml</t>
         </is>
       </c>
       <c r="C289" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - SU</t>
+          <t>Prodotto - More Inside</t>
         </is>
       </c>
       <c r="D289" s="6" t="n">
-        <v>25.4</v>
+        <v>25.5</v>
       </c>
       <c r="E289" s="5" t="n"/>
     </row>
@@ -6138,7 +6138,7 @@
       </c>
       <c r="B290" s="5" t="inlineStr">
         <is>
-          <t>SU/Aftersun 150 ml</t>
+          <t>SU/Hair &amp; Body Wash 75 ml</t>
         </is>
       </c>
       <c r="C290" s="5" t="inlineStr">
@@ -6147,7 +6147,7 @@
         </is>
       </c>
       <c r="D290" s="6" t="n">
-        <v>25.4</v>
+        <v>9.4</v>
       </c>
       <c r="E290" s="5" t="n"/>
     </row>
@@ -6157,7 +6157,7 @@
       </c>
       <c r="B291" s="5" t="inlineStr">
         <is>
-          <t>SU/Conscious Sunscreen SPF 30 100 ml</t>
+          <t>SU/Hair &amp; Body Wash 500 ml</t>
         </is>
       </c>
       <c r="C291" s="5" t="inlineStr">
@@ -6166,7 +6166,7 @@
         </is>
       </c>
       <c r="D291" s="6" t="n">
-        <v>30.5</v>
+        <v>36</v>
       </c>
       <c r="E291" s="5" t="n"/>
     </row>
@@ -6176,16 +6176,16 @@
       </c>
       <c r="B292" s="5" t="inlineStr">
         <is>
-          <t>Reinforcing Bodifying Fluid 50 ml</t>
+          <t>SU/Hair Mask 150 ml</t>
         </is>
       </c>
       <c r="C292" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Liquid Spell</t>
+          <t>Prodotto - SU</t>
         </is>
       </c>
       <c r="D292" s="6" t="n">
-        <v>23.2</v>
+        <v>22.4</v>
       </c>
       <c r="E292" s="5" t="n"/>
     </row>
@@ -6195,16 +6195,16 @@
       </c>
       <c r="B293" s="5" t="inlineStr">
         <is>
-          <t>Reinforcing Bodifying Fluid 125 ml</t>
+          <t>SU/Hair Milk 50 ml</t>
         </is>
       </c>
       <c r="C293" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Liquid Spell</t>
+          <t>Prodotto - SU</t>
         </is>
       </c>
       <c r="D293" s="6" t="n">
-        <v>40.9</v>
+        <v>14</v>
       </c>
       <c r="E293" s="5" t="n"/>
     </row>
@@ -6214,16 +6214,16 @@
       </c>
       <c r="B294" s="5" t="inlineStr">
         <is>
-          <t>Hair Refresher - Shampoo a Secco 150 ml</t>
+          <t>SU/Hair Milk 135 ml</t>
         </is>
       </c>
       <c r="C294" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Hair Refresher</t>
+          <t>Prodotto - SU</t>
         </is>
       </c>
       <c r="D294" s="6" t="n">
-        <v>27.8</v>
+        <v>22.4</v>
       </c>
       <c r="E294" s="5" t="n"/>
     </row>
@@ -6233,16 +6233,16 @@
       </c>
       <c r="B295" s="5" t="inlineStr">
         <is>
-          <t>Hand Sanitizer 75 ml</t>
+          <t>SU/Tan Maximizer 150 ml</t>
         </is>
       </c>
       <c r="C295" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Gel del Buon Auspicio</t>
+          <t>Prodotto - SU</t>
         </is>
       </c>
       <c r="D295" s="6" t="n">
-        <v>6</v>
+        <v>25.4</v>
       </c>
       <c r="E295" s="5" t="n"/>
     </row>
@@ -6252,16 +6252,16 @@
       </c>
       <c r="B296" s="5" t="inlineStr">
         <is>
-          <t>Nettare Lavante 280 ml</t>
+          <t>SU/Aftersun 150 ml</t>
         </is>
       </c>
       <c r="C296" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Authentic Formulas</t>
+          <t>Prodotto - SU</t>
         </is>
       </c>
       <c r="D296" s="6" t="n">
-        <v>26.4</v>
+        <v>25.4</v>
       </c>
       <c r="E296" s="5" t="n"/>
     </row>
@@ -6271,16 +6271,16 @@
       </c>
       <c r="B297" s="5" t="inlineStr">
         <is>
-          <t>Balsamo Idratante 150 ml</t>
+          <t>SU/Conscious Sunscreen SPF 30 100 ml</t>
         </is>
       </c>
       <c r="C297" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Authentic Formulas</t>
+          <t>Prodotto - SU</t>
         </is>
       </c>
       <c r="D297" s="6" t="n">
-        <v>24.9</v>
+        <v>30.5</v>
       </c>
       <c r="E297" s="5" t="n"/>
     </row>
@@ -6290,16 +6290,16 @@
       </c>
       <c r="B298" s="5" t="inlineStr">
         <is>
-          <t>Burro Restitutivo 200 ml</t>
+          <t>Reinforcing Bodifying Fluid 50 ml</t>
         </is>
       </c>
       <c r="C298" s="5" t="inlineStr">
         <is>
-          <t>Prodotto - Authentic Formulas</t>
+          <t>Prodotto - Liquid Spell</t>
         </is>
       </c>
       <c r="D298" s="6" t="n">
-        <v>33.3</v>
+        <v>23.2</v>
       </c>
       <c r="E298" s="5" t="n"/>
     </row>
@@ -6309,18 +6309,132 @@
       </c>
       <c r="B299" s="5" t="inlineStr">
         <is>
+          <t>Reinforcing Bodifying Fluid 125 ml</t>
+        </is>
+      </c>
+      <c r="C299" s="5" t="inlineStr">
+        <is>
+          <t>Prodotto - Liquid Spell</t>
+        </is>
+      </c>
+      <c r="D299" s="6" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="E299" s="5" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="5" t="n">
+        <v>299</v>
+      </c>
+      <c r="B300" s="5" t="inlineStr">
+        <is>
+          <t>Hair Refresher - Shampoo a Secco 150 ml</t>
+        </is>
+      </c>
+      <c r="C300" s="5" t="inlineStr">
+        <is>
+          <t>Prodotto - Hair Refresher</t>
+        </is>
+      </c>
+      <c r="D300" s="6" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="E300" s="5" t="n"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="B301" s="5" t="inlineStr">
+        <is>
+          <t>Hand Sanitizer 75 ml</t>
+        </is>
+      </c>
+      <c r="C301" s="5" t="inlineStr">
+        <is>
+          <t>Prodotto - Gel del Buon Auspicio</t>
+        </is>
+      </c>
+      <c r="D301" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E301" s="5" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="5" t="n">
+        <v>301</v>
+      </c>
+      <c r="B302" s="5" t="inlineStr">
+        <is>
+          <t>Nettare Lavante 280 ml</t>
+        </is>
+      </c>
+      <c r="C302" s="5" t="inlineStr">
+        <is>
+          <t>Prodotto - Authentic Formulas</t>
+        </is>
+      </c>
+      <c r="D302" s="6" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="E302" s="5" t="n"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="5" t="n">
+        <v>302</v>
+      </c>
+      <c r="B303" s="5" t="inlineStr">
+        <is>
+          <t>Balsamo Idratante 150 ml</t>
+        </is>
+      </c>
+      <c r="C303" s="5" t="inlineStr">
+        <is>
+          <t>Prodotto - Authentic Formulas</t>
+        </is>
+      </c>
+      <c r="D303" s="6" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="E303" s="5" t="n"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="5" t="n">
+        <v>303</v>
+      </c>
+      <c r="B304" s="5" t="inlineStr">
+        <is>
+          <t>Burro Restitutivo 200 ml</t>
+        </is>
+      </c>
+      <c r="C304" s="5" t="inlineStr">
+        <is>
+          <t>Prodotto - Authentic Formulas</t>
+        </is>
+      </c>
+      <c r="D304" s="6" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="E304" s="5" t="n"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="5" t="n">
+        <v>304</v>
+      </c>
+      <c r="B305" s="5" t="inlineStr">
+        <is>
           <t>Olio Nutriente 140 ml</t>
         </is>
       </c>
-      <c r="C299" s="5" t="inlineStr">
+      <c r="C305" s="5" t="inlineStr">
         <is>
           <t>Prodotto - Authentic Formulas</t>
         </is>
       </c>
-      <c r="D299" s="6" t="n">
+      <c r="D305" s="6" t="n">
         <v>43.5</v>
       </c>
-      <c r="E299" s="5" t="n"/>
+      <c r="E305" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11417,7 +11531,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Scegli una voce dal menu, oppure aggiungila prima nel foglio Listino." type="list">
-      <formula1>=Listino!$B$2:$B$299</formula1>
+      <formula1>=Listino!$B$2:$B$305</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Contanti,Carta,Satispay,Altro"</formula1>

</xml_diff>